<commit_message>
VAT Data: prepare R script
- R script prepared for input data
- Wait for properly formatted threshold and rate spreadsheets
</commit_message>
<xml_diff>
--- a/source_data/oecd_vat_gst_rates_ctt_trends.xlsx
+++ b/source_data/oecd_vat_gst_rates_ctt_trends.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\international-tax-competitiveness-index\source_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33CD44B2-8A28-4DE1-969D-148181012E50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27E2BE37-5B82-44E7-BF95-47BE14842A5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -911,19 +911,19 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -932,8 +932,8 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -950,10 +950,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1219,45 +1215,46 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W64"/>
+  <dimension ref="A1:X64"/>
   <sheetFormatPr defaultColWidth="9.06640625" defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="15" width="0" hidden="1" customWidth="1"/>
     <col min="18" max="18" width="8.1328125" customWidth="1"/>
-    <col min="19" max="21" width="4.86328125" customWidth="1"/>
-    <col min="22" max="22" width="10.86328125" customWidth="1"/>
-    <col min="23" max="23" width="15.3984375" customWidth="1"/>
+    <col min="19" max="22" width="4.86328125" customWidth="1"/>
+    <col min="23" max="23" width="10.86328125" customWidth="1"/>
+    <col min="24" max="24" width="15.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="14.65" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="22" t="s">
+    <row r="1" spans="1:24" ht="14.65" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="22"/>
-      <c r="M1" s="22"/>
-      <c r="N1" s="22"/>
-      <c r="O1" s="22"/>
-      <c r="P1" s="22"/>
-      <c r="Q1" s="22"/>
-      <c r="R1" s="22"/>
-      <c r="S1" s="22"/>
-      <c r="T1" s="22"/>
-      <c r="U1" s="22"/>
-      <c r="V1" s="22"/>
-      <c r="W1" s="22"/>
-    </row>
-    <row r="2" spans="1:23" ht="50.1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="21"/>
+      <c r="O1" s="21"/>
+      <c r="P1" s="21"/>
+      <c r="Q1" s="21"/>
+      <c r="R1" s="21"/>
+      <c r="S1" s="21"/>
+      <c r="T1" s="21"/>
+      <c r="U1" s="21"/>
+      <c r="V1" s="21"/>
+      <c r="W1" s="21"/>
+      <c r="X1" s="21"/>
+    </row>
+    <row r="2" spans="1:24" ht="50.1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B2" s="12">
         <v>2005</v>
       </c>
@@ -1318,14 +1315,17 @@
       <c r="U2" s="12">
         <v>2025</v>
       </c>
-      <c r="V2" s="18" t="s">
+      <c r="V2" s="12">
+        <v>2026</v>
+      </c>
+      <c r="W2" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="W2" s="16" t="s">
+      <c r="X2" s="16" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -1389,14 +1389,15 @@
       <c r="U3" s="9">
         <v>10</v>
       </c>
-      <c r="V3" s="13">
+      <c r="V3" s="9"/>
+      <c r="W3" s="13">
         <v>0</v>
       </c>
-      <c r="W3" s="13" t="s">
+      <c r="X3" s="13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>26</v>
       </c>
@@ -1460,14 +1461,15 @@
       <c r="U4" s="10">
         <v>20</v>
       </c>
-      <c r="V4" s="14" t="s">
+      <c r="V4" s="10"/>
+      <c r="W4" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="W4" s="14">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X4" s="14">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>49</v>
       </c>
@@ -1531,14 +1533,15 @@
       <c r="U5" s="11">
         <v>21</v>
       </c>
-      <c r="V5" s="15" t="s">
+      <c r="V5" s="11"/>
+      <c r="W5" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="W5" s="15" t="s">
+      <c r="X5" s="15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>27</v>
       </c>
@@ -1602,14 +1605,15 @@
       <c r="U6" s="10">
         <v>5</v>
       </c>
-      <c r="V6" s="14">
+      <c r="V6" s="10"/>
+      <c r="W6" s="14">
         <v>0</v>
       </c>
-      <c r="W6" s="14" t="s">
+      <c r="X6" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>1</v>
       </c>
@@ -1673,14 +1677,15 @@
       <c r="U7" s="11">
         <v>19</v>
       </c>
-      <c r="V7" s="15" t="s">
-        <v>12</v>
-      </c>
+      <c r="V7" s="11"/>
       <c r="W7" s="15" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X7" s="15" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>43</v>
       </c>
@@ -1744,14 +1749,15 @@
       <c r="U8" s="10">
         <v>19</v>
       </c>
-      <c r="V8" s="14" t="s">
+      <c r="V8" s="10"/>
+      <c r="W8" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="W8" s="14" t="s">
+      <c r="X8" s="14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>44</v>
       </c>
@@ -1803,12 +1809,13 @@
       <c r="U9" s="11">
         <v>13</v>
       </c>
-      <c r="V9" s="15" t="s">
+      <c r="V9" s="11"/>
+      <c r="W9" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="W9" s="15"/>
-    </row>
-    <row r="10" spans="1:23" ht="15.95" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="X9" s="15"/>
+    </row>
+    <row r="10" spans="1:24" ht="15.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>53</v>
       </c>
@@ -1872,14 +1879,15 @@
       <c r="U10" s="10">
         <v>21</v>
       </c>
-      <c r="V10" s="14" t="s">
+      <c r="V10" s="10"/>
+      <c r="W10" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="W10" s="14" t="s">
+      <c r="X10" s="14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>54</v>
       </c>
@@ -1943,14 +1951,15 @@
       <c r="U11" s="11">
         <v>25</v>
       </c>
-      <c r="V11" s="15">
+      <c r="V11" s="11"/>
+      <c r="W11" s="15">
         <v>0</v>
       </c>
-      <c r="W11" s="15" t="s">
+      <c r="X11" s="15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>51</v>
       </c>
@@ -2014,14 +2023,15 @@
       <c r="U12" s="10">
         <v>24</v>
       </c>
-      <c r="V12" s="14" t="s">
+      <c r="V12" s="10"/>
+      <c r="W12" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="W12" s="14" t="s">
+      <c r="X12" s="14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>55</v>
       </c>
@@ -2085,14 +2095,15 @@
       <c r="U13" s="11">
         <v>25.5</v>
       </c>
-      <c r="V13" s="15" t="s">
+      <c r="V13" s="11"/>
+      <c r="W13" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="W13" s="15" t="s">
+      <c r="X13" s="15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="22.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:24" ht="22.5" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>28</v>
       </c>
@@ -2156,14 +2167,15 @@
       <c r="U14" s="10">
         <v>20</v>
       </c>
-      <c r="V14" s="14" t="s">
+      <c r="V14" s="10"/>
+      <c r="W14" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="W14" s="14" t="s">
+      <c r="X14" s="14" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>29</v>
       </c>
@@ -2227,14 +2239,15 @@
       <c r="U15" s="11">
         <v>19</v>
       </c>
-      <c r="V15" s="15" t="s">
+      <c r="V15" s="11"/>
+      <c r="W15" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="W15" s="15" t="s">
+      <c r="X15" s="15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>30</v>
       </c>
@@ -2298,14 +2311,15 @@
       <c r="U16" s="10">
         <v>24</v>
       </c>
-      <c r="V16" s="14" t="s">
+      <c r="V16" s="10"/>
+      <c r="W16" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="W16" s="14" t="s">
+      <c r="X16" s="14" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
         <v>56</v>
       </c>
@@ -2369,14 +2383,15 @@
       <c r="U17" s="11">
         <v>27</v>
       </c>
-      <c r="V17" s="15" t="s">
+      <c r="V17" s="11"/>
+      <c r="W17" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="W17" s="15" t="s">
+      <c r="X17" s="15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>2</v>
       </c>
@@ -2440,14 +2455,15 @@
       <c r="U18" s="10">
         <v>24</v>
       </c>
-      <c r="V18" s="14" t="s">
-        <v>19</v>
-      </c>
+      <c r="V18" s="10"/>
       <c r="W18" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="X18" s="14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
         <v>31</v>
       </c>
@@ -2511,14 +2527,15 @@
       <c r="U19" s="11">
         <v>23</v>
       </c>
-      <c r="V19" s="15" t="s">
-        <v>20</v>
-      </c>
+      <c r="V19" s="11"/>
       <c r="W19" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="X19" s="15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>32</v>
       </c>
@@ -2582,14 +2599,15 @@
       <c r="U20" s="10">
         <v>18</v>
       </c>
-      <c r="V20" s="14">
-        <v>0</v>
-      </c>
+      <c r="V20" s="10"/>
       <c r="W20" s="14">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="X20" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
         <v>57</v>
       </c>
@@ -2653,14 +2671,15 @@
       <c r="U21" s="11">
         <v>22</v>
       </c>
-      <c r="V21" s="15" t="s">
-        <v>21</v>
-      </c>
+      <c r="V21" s="11"/>
       <c r="W21" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="X21" s="15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>42</v>
       </c>
@@ -2724,14 +2743,15 @@
       <c r="U22" s="10">
         <v>10</v>
       </c>
-      <c r="V22" s="14">
+      <c r="V22" s="10"/>
+      <c r="W22" s="14">
         <v>8</v>
       </c>
-      <c r="W22" s="14" t="s">
+      <c r="X22" s="14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
         <v>3</v>
       </c>
@@ -2795,14 +2815,15 @@
       <c r="U23" s="11">
         <v>10</v>
       </c>
-      <c r="V23" s="15">
+      <c r="V23" s="11"/>
+      <c r="W23" s="15">
         <v>0</v>
       </c>
-      <c r="W23" s="15" t="s">
+      <c r="X23" s="15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>33</v>
       </c>
@@ -2866,14 +2887,15 @@
       <c r="U24" s="10">
         <v>21</v>
       </c>
-      <c r="V24" s="10" t="s">
+      <c r="V24" s="10"/>
+      <c r="W24" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="W24" s="14" t="s">
+      <c r="X24" s="14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
         <v>34</v>
       </c>
@@ -2937,14 +2959,15 @@
       <c r="U25" s="11">
         <v>21</v>
       </c>
-      <c r="V25" s="15" t="s">
+      <c r="V25" s="11"/>
+      <c r="W25" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="W25" s="15" t="s">
+      <c r="X25" s="15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>35</v>
       </c>
@@ -3008,14 +3031,15 @@
       <c r="U26" s="10">
         <v>17</v>
       </c>
-      <c r="V26" s="14" t="s">
-        <v>23</v>
-      </c>
+      <c r="V26" s="10"/>
       <c r="W26" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="X26" s="14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
         <v>36</v>
       </c>
@@ -3079,14 +3103,15 @@
       <c r="U27" s="11">
         <v>16</v>
       </c>
-      <c r="V27" s="15">
+      <c r="V27" s="11"/>
+      <c r="W27" s="15">
         <v>0</v>
       </c>
-      <c r="W27" s="15">
+      <c r="X27" s="15">
         <v>8</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>58</v>
       </c>
@@ -3150,14 +3175,15 @@
       <c r="U28" s="10">
         <v>21</v>
       </c>
-      <c r="V28" s="14">
+      <c r="V28" s="10"/>
+      <c r="W28" s="14">
         <v>9</v>
       </c>
-      <c r="W28" s="14" t="s">
+      <c r="X28" s="14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
         <v>4</v>
       </c>
@@ -3221,14 +3247,15 @@
       <c r="U29" s="11">
         <v>15</v>
       </c>
-      <c r="V29" s="15">
+      <c r="V29" s="11"/>
+      <c r="W29" s="15">
         <v>0</v>
       </c>
-      <c r="W29" s="15" t="s">
+      <c r="X29" s="15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>37</v>
       </c>
@@ -3292,14 +3319,15 @@
       <c r="U30" s="10">
         <v>25</v>
       </c>
-      <c r="V30" s="10" t="s">
+      <c r="V30" s="10"/>
+      <c r="W30" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="W30" s="14" t="s">
+      <c r="X30" s="14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
         <v>59</v>
       </c>
@@ -3363,14 +3391,15 @@
       <c r="U31" s="11">
         <v>23</v>
       </c>
-      <c r="V31" s="15" t="s">
+      <c r="V31" s="11"/>
+      <c r="W31" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="W31" s="15" t="s">
+      <c r="X31" s="15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>38</v>
       </c>
@@ -3434,14 +3463,15 @@
       <c r="U32" s="10">
         <v>23</v>
       </c>
-      <c r="V32" s="14" t="s">
+      <c r="V32" s="10"/>
+      <c r="W32" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="W32" s="14" t="s">
+      <c r="X32" s="14" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
         <v>39</v>
       </c>
@@ -3505,14 +3535,15 @@
       <c r="U33" s="11">
         <v>23</v>
       </c>
-      <c r="V33" s="26" t="s">
+      <c r="V33" s="11"/>
+      <c r="W33" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="W33" s="15" t="s">
+      <c r="X33" s="15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>52</v>
       </c>
@@ -3576,14 +3607,15 @@
       <c r="U34" s="10">
         <v>22</v>
       </c>
-      <c r="V34" s="14" t="s">
-        <v>25</v>
-      </c>
+      <c r="V34" s="10"/>
       <c r="W34" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="X34" s="14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="35" spans="1:23" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:24" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
         <v>40</v>
       </c>
@@ -3647,14 +3679,15 @@
       <c r="U35" s="11">
         <v>21</v>
       </c>
-      <c r="V35" s="15" t="s">
+      <c r="V35" s="11"/>
+      <c r="W35" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="W35" s="15" t="s">
+      <c r="X35" s="15" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="36" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>41</v>
       </c>
@@ -3718,14 +3751,15 @@
       <c r="U36" s="10">
         <v>25</v>
       </c>
-      <c r="V36" s="14" t="s">
+      <c r="V36" s="10"/>
+      <c r="W36" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="W36" s="14" t="s">
+      <c r="X36" s="14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="37" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
         <v>60</v>
       </c>
@@ -3789,14 +3823,15 @@
       <c r="U37" s="11">
         <v>8.1</v>
       </c>
-      <c r="V37" s="15" t="s">
+      <c r="V37" s="11"/>
+      <c r="W37" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="W37" s="15" t="s">
+      <c r="X37" s="15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="38" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>45</v>
       </c>
@@ -3860,14 +3895,15 @@
       <c r="U38" s="10">
         <v>20</v>
       </c>
-      <c r="V38" s="14" t="s">
+      <c r="V38" s="10"/>
+      <c r="W38" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="W38" s="14" t="s">
+      <c r="X38" s="14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="39" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
         <v>61</v>
       </c>
@@ -3931,14 +3967,15 @@
       <c r="U39" s="11">
         <v>20</v>
       </c>
-      <c r="V39" s="15" t="s">
+      <c r="V39" s="11"/>
+      <c r="W39" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="W39" s="15" t="s">
+      <c r="X39" s="15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="40" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="6" t="s">
         <v>7</v>
       </c>
@@ -4015,10 +4052,11 @@
         <f>AVERAGE(U3:U39)</f>
         <v>19.475675675675678</v>
       </c>
-      <c r="V40" s="8"/>
-      <c r="W40" s="17"/>
-    </row>
-    <row r="41" spans="1:23" ht="17.45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="V40" s="7"/>
+      <c r="W40" s="8"/>
+      <c r="X40" s="17"/>
+    </row>
+    <row r="41" spans="1:24" ht="17.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="25" t="s">
         <v>76</v>
       </c>
@@ -4042,34 +4080,36 @@
       <c r="S41" s="3"/>
       <c r="T41" s="3"/>
       <c r="U41" s="3"/>
-    </row>
-    <row r="42" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A42" s="23" t="s">
+      <c r="V41" s="3"/>
+    </row>
+    <row r="42" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A42" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="B42" s="20"/>
-      <c r="C42" s="20"/>
-      <c r="D42" s="20"/>
-      <c r="E42" s="20"/>
-      <c r="F42" s="20"/>
-      <c r="G42" s="20"/>
-      <c r="H42" s="20"/>
-      <c r="I42" s="20"/>
-      <c r="J42" s="20"/>
-      <c r="K42" s="20"/>
-      <c r="L42" s="20"/>
-      <c r="M42" s="20"/>
-      <c r="N42" s="20"/>
-      <c r="O42" s="20"/>
-      <c r="P42" s="20"/>
-      <c r="Q42" s="20"/>
+      <c r="B42" s="23"/>
+      <c r="C42" s="23"/>
+      <c r="D42" s="23"/>
+      <c r="E42" s="23"/>
+      <c r="F42" s="23"/>
+      <c r="G42" s="23"/>
+      <c r="H42" s="23"/>
+      <c r="I42" s="23"/>
+      <c r="J42" s="23"/>
+      <c r="K42" s="23"/>
+      <c r="L42" s="23"/>
+      <c r="M42" s="23"/>
+      <c r="N42" s="23"/>
+      <c r="O42" s="23"/>
+      <c r="P42" s="23"/>
+      <c r="Q42" s="23"/>
       <c r="R42" s="4"/>
       <c r="S42" s="4"/>
       <c r="T42" s="4"/>
       <c r="U42" s="4"/>
-    </row>
-    <row r="43" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A43" s="20" t="s">
+      <c r="V42" s="4"/>
+    </row>
+    <row r="43" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A43" s="23" t="s">
         <v>9</v>
       </c>
       <c r="B43" s="24"/>
@@ -4092,526 +4132,545 @@
       <c r="S43" s="5"/>
       <c r="T43" s="5"/>
       <c r="U43" s="5"/>
-    </row>
-    <row r="44" spans="1:23" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="19" t="s">
+      <c r="V43" s="5"/>
+    </row>
+    <row r="44" spans="1:24" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="B44" s="19"/>
-      <c r="C44" s="19"/>
-      <c r="D44" s="19"/>
-      <c r="E44" s="19"/>
-      <c r="F44" s="19"/>
-      <c r="G44" s="19"/>
-      <c r="H44" s="19"/>
-      <c r="I44" s="19"/>
-      <c r="J44" s="19"/>
-      <c r="K44" s="19"/>
-      <c r="L44" s="19"/>
-      <c r="M44" s="19"/>
-      <c r="N44" s="19"/>
-      <c r="O44" s="19"/>
-      <c r="P44" s="19"/>
-      <c r="Q44" s="19"/>
-      <c r="R44" s="19"/>
-      <c r="S44" s="19"/>
-      <c r="T44" s="19"/>
-      <c r="U44" s="19"/>
-      <c r="V44" s="19"/>
-      <c r="W44" s="19"/>
-    </row>
-    <row r="45" spans="1:23" ht="53.45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="19" t="s">
+      <c r="B44" s="20"/>
+      <c r="C44" s="20"/>
+      <c r="D44" s="20"/>
+      <c r="E44" s="20"/>
+      <c r="F44" s="20"/>
+      <c r="G44" s="20"/>
+      <c r="H44" s="20"/>
+      <c r="I44" s="20"/>
+      <c r="J44" s="20"/>
+      <c r="K44" s="20"/>
+      <c r="L44" s="20"/>
+      <c r="M44" s="20"/>
+      <c r="N44" s="20"/>
+      <c r="O44" s="20"/>
+      <c r="P44" s="20"/>
+      <c r="Q44" s="20"/>
+      <c r="R44" s="20"/>
+      <c r="S44" s="20"/>
+      <c r="T44" s="20"/>
+      <c r="U44" s="20"/>
+      <c r="V44" s="20"/>
+      <c r="W44" s="20"/>
+      <c r="X44" s="20"/>
+    </row>
+    <row r="45" spans="1:24" ht="53.45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="B45" s="19"/>
-      <c r="C45" s="19"/>
-      <c r="D45" s="19"/>
-      <c r="E45" s="19"/>
-      <c r="F45" s="19"/>
-      <c r="G45" s="19"/>
-      <c r="H45" s="19"/>
-      <c r="I45" s="19"/>
-      <c r="J45" s="19"/>
-      <c r="K45" s="19"/>
-      <c r="L45" s="19"/>
-      <c r="M45" s="19"/>
-      <c r="N45" s="19"/>
-      <c r="O45" s="19"/>
-      <c r="P45" s="19"/>
-      <c r="Q45" s="19"/>
-      <c r="R45" s="19"/>
-      <c r="S45" s="19"/>
-      <c r="T45" s="19"/>
-      <c r="U45" s="19"/>
-      <c r="V45" s="19"/>
-      <c r="W45" s="19"/>
-    </row>
-    <row r="46" spans="1:23" ht="15.6" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="19"/>
-      <c r="B46" s="19"/>
-      <c r="C46" s="19"/>
-      <c r="D46" s="19"/>
-      <c r="E46" s="19"/>
-      <c r="F46" s="19"/>
-      <c r="G46" s="19"/>
-      <c r="H46" s="19"/>
-      <c r="I46" s="19"/>
-      <c r="J46" s="19"/>
-      <c r="K46" s="19"/>
-      <c r="L46" s="19"/>
-      <c r="M46" s="19"/>
-      <c r="N46" s="19"/>
-      <c r="O46" s="19"/>
-      <c r="P46" s="19"/>
-      <c r="Q46" s="19"/>
-      <c r="R46" s="19"/>
-      <c r="S46" s="19"/>
-      <c r="T46" s="19"/>
-      <c r="U46" s="19"/>
-      <c r="V46" s="19"/>
-      <c r="W46" s="19"/>
-    </row>
-    <row r="47" spans="1:23" ht="15.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="19"/>
-      <c r="B47" s="19"/>
-      <c r="C47" s="19"/>
-      <c r="D47" s="19"/>
-      <c r="E47" s="19"/>
-      <c r="F47" s="19"/>
-      <c r="G47" s="19"/>
-      <c r="H47" s="19"/>
-      <c r="I47" s="19"/>
-      <c r="J47" s="19"/>
-      <c r="K47" s="19"/>
-      <c r="L47" s="19"/>
-      <c r="M47" s="19"/>
-      <c r="N47" s="19"/>
-      <c r="O47" s="19"/>
-      <c r="P47" s="19"/>
-      <c r="Q47" s="19"/>
-      <c r="R47" s="19"/>
-      <c r="S47" s="19"/>
-      <c r="T47" s="19"/>
-      <c r="U47" s="19"/>
-      <c r="V47" s="19"/>
-      <c r="W47" s="19"/>
-    </row>
-    <row r="48" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A48" s="20" t="s">
+      <c r="B45" s="20"/>
+      <c r="C45" s="20"/>
+      <c r="D45" s="20"/>
+      <c r="E45" s="20"/>
+      <c r="F45" s="20"/>
+      <c r="G45" s="20"/>
+      <c r="H45" s="20"/>
+      <c r="I45" s="20"/>
+      <c r="J45" s="20"/>
+      <c r="K45" s="20"/>
+      <c r="L45" s="20"/>
+      <c r="M45" s="20"/>
+      <c r="N45" s="20"/>
+      <c r="O45" s="20"/>
+      <c r="P45" s="20"/>
+      <c r="Q45" s="20"/>
+      <c r="R45" s="20"/>
+      <c r="S45" s="20"/>
+      <c r="T45" s="20"/>
+      <c r="U45" s="20"/>
+      <c r="V45" s="20"/>
+      <c r="W45" s="20"/>
+      <c r="X45" s="20"/>
+    </row>
+    <row r="46" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="20"/>
+      <c r="B46" s="20"/>
+      <c r="C46" s="20"/>
+      <c r="D46" s="20"/>
+      <c r="E46" s="20"/>
+      <c r="F46" s="20"/>
+      <c r="G46" s="20"/>
+      <c r="H46" s="20"/>
+      <c r="I46" s="20"/>
+      <c r="J46" s="20"/>
+      <c r="K46" s="20"/>
+      <c r="L46" s="20"/>
+      <c r="M46" s="20"/>
+      <c r="N46" s="20"/>
+      <c r="O46" s="20"/>
+      <c r="P46" s="20"/>
+      <c r="Q46" s="20"/>
+      <c r="R46" s="20"/>
+      <c r="S46" s="20"/>
+      <c r="T46" s="20"/>
+      <c r="U46" s="20"/>
+      <c r="V46" s="20"/>
+      <c r="W46" s="20"/>
+      <c r="X46" s="20"/>
+    </row>
+    <row r="47" spans="1:24" ht="15.95" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="20"/>
+      <c r="B47" s="20"/>
+      <c r="C47" s="20"/>
+      <c r="D47" s="20"/>
+      <c r="E47" s="20"/>
+      <c r="F47" s="20"/>
+      <c r="G47" s="20"/>
+      <c r="H47" s="20"/>
+      <c r="I47" s="20"/>
+      <c r="J47" s="20"/>
+      <c r="K47" s="20"/>
+      <c r="L47" s="20"/>
+      <c r="M47" s="20"/>
+      <c r="N47" s="20"/>
+      <c r="O47" s="20"/>
+      <c r="P47" s="20"/>
+      <c r="Q47" s="20"/>
+      <c r="R47" s="20"/>
+      <c r="S47" s="20"/>
+      <c r="T47" s="20"/>
+      <c r="U47" s="20"/>
+      <c r="V47" s="20"/>
+      <c r="W47" s="20"/>
+      <c r="X47" s="20"/>
+    </row>
+    <row r="48" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A48" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="B48" s="20"/>
+      <c r="B48" s="23"/>
       <c r="C48" s="4"/>
     </row>
-    <row r="49" spans="1:23" ht="24.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="19" t="s">
+    <row r="49" spans="1:24" ht="24.95" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A49" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="B49" s="19"/>
-      <c r="C49" s="19"/>
-      <c r="D49" s="19"/>
-      <c r="E49" s="19"/>
-      <c r="F49" s="19"/>
-      <c r="G49" s="19"/>
-      <c r="H49" s="19"/>
-      <c r="I49" s="19"/>
-      <c r="J49" s="19"/>
-      <c r="K49" s="19"/>
-      <c r="L49" s="19"/>
-      <c r="M49" s="19"/>
-      <c r="N49" s="19"/>
-      <c r="O49" s="19"/>
-      <c r="P49" s="19"/>
-      <c r="Q49" s="19"/>
-      <c r="R49" s="19"/>
-      <c r="S49" s="19"/>
-      <c r="T49" s="19"/>
-      <c r="U49" s="19"/>
-      <c r="V49" s="19"/>
-      <c r="W49" s="19"/>
-    </row>
-    <row r="50" spans="1:23" ht="68.45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="19" t="s">
+      <c r="B49" s="20"/>
+      <c r="C49" s="20"/>
+      <c r="D49" s="20"/>
+      <c r="E49" s="20"/>
+      <c r="F49" s="20"/>
+      <c r="G49" s="20"/>
+      <c r="H49" s="20"/>
+      <c r="I49" s="20"/>
+      <c r="J49" s="20"/>
+      <c r="K49" s="20"/>
+      <c r="L49" s="20"/>
+      <c r="M49" s="20"/>
+      <c r="N49" s="20"/>
+      <c r="O49" s="20"/>
+      <c r="P49" s="20"/>
+      <c r="Q49" s="20"/>
+      <c r="R49" s="20"/>
+      <c r="S49" s="20"/>
+      <c r="T49" s="20"/>
+      <c r="U49" s="20"/>
+      <c r="V49" s="20"/>
+      <c r="W49" s="20"/>
+      <c r="X49" s="20"/>
+    </row>
+    <row r="50" spans="1:24" ht="68.45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A50" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="B50" s="19"/>
-      <c r="C50" s="19"/>
-      <c r="D50" s="19"/>
-      <c r="E50" s="19"/>
-      <c r="F50" s="19"/>
-      <c r="G50" s="19"/>
-      <c r="H50" s="19"/>
-      <c r="I50" s="19"/>
-      <c r="J50" s="19"/>
-      <c r="K50" s="19"/>
-      <c r="L50" s="19"/>
-      <c r="M50" s="19"/>
-      <c r="N50" s="19"/>
-      <c r="O50" s="19"/>
-      <c r="P50" s="19"/>
-      <c r="Q50" s="19"/>
-      <c r="R50" s="19"/>
-      <c r="S50" s="19"/>
-      <c r="T50" s="19"/>
-      <c r="U50" s="19"/>
-      <c r="V50" s="19"/>
-      <c r="W50" s="19"/>
-    </row>
-    <row r="51" spans="1:23" ht="54" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="19" t="s">
+      <c r="B50" s="20"/>
+      <c r="C50" s="20"/>
+      <c r="D50" s="20"/>
+      <c r="E50" s="20"/>
+      <c r="F50" s="20"/>
+      <c r="G50" s="20"/>
+      <c r="H50" s="20"/>
+      <c r="I50" s="20"/>
+      <c r="J50" s="20"/>
+      <c r="K50" s="20"/>
+      <c r="L50" s="20"/>
+      <c r="M50" s="20"/>
+      <c r="N50" s="20"/>
+      <c r="O50" s="20"/>
+      <c r="P50" s="20"/>
+      <c r="Q50" s="20"/>
+      <c r="R50" s="20"/>
+      <c r="S50" s="20"/>
+      <c r="T50" s="20"/>
+      <c r="U50" s="20"/>
+      <c r="V50" s="20"/>
+      <c r="W50" s="20"/>
+      <c r="X50" s="20"/>
+    </row>
+    <row r="51" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A51" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="B51" s="19"/>
-      <c r="C51" s="19"/>
-      <c r="D51" s="19"/>
-      <c r="E51" s="19"/>
-      <c r="F51" s="19"/>
-      <c r="G51" s="19"/>
-      <c r="H51" s="19"/>
-      <c r="I51" s="19"/>
-      <c r="J51" s="19"/>
-      <c r="K51" s="19"/>
-      <c r="L51" s="19"/>
-      <c r="M51" s="19"/>
-      <c r="N51" s="19"/>
-      <c r="O51" s="19"/>
-      <c r="P51" s="19"/>
-      <c r="Q51" s="19"/>
-      <c r="R51" s="19"/>
-      <c r="S51" s="19"/>
-      <c r="T51" s="19"/>
-      <c r="U51" s="19"/>
-      <c r="V51" s="19"/>
-      <c r="W51" s="19"/>
-    </row>
-    <row r="52" spans="1:23" ht="26.45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="19" t="s">
+      <c r="B51" s="20"/>
+      <c r="C51" s="20"/>
+      <c r="D51" s="20"/>
+      <c r="E51" s="20"/>
+      <c r="F51" s="20"/>
+      <c r="G51" s="20"/>
+      <c r="H51" s="20"/>
+      <c r="I51" s="20"/>
+      <c r="J51" s="20"/>
+      <c r="K51" s="20"/>
+      <c r="L51" s="20"/>
+      <c r="M51" s="20"/>
+      <c r="N51" s="20"/>
+      <c r="O51" s="20"/>
+      <c r="P51" s="20"/>
+      <c r="Q51" s="20"/>
+      <c r="R51" s="20"/>
+      <c r="S51" s="20"/>
+      <c r="T51" s="20"/>
+      <c r="U51" s="20"/>
+      <c r="V51" s="20"/>
+      <c r="W51" s="20"/>
+      <c r="X51" s="20"/>
+    </row>
+    <row r="52" spans="1:24" ht="26.45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A52" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="B52" s="19"/>
-      <c r="C52" s="19"/>
-      <c r="D52" s="19"/>
-      <c r="E52" s="19"/>
-      <c r="F52" s="19"/>
-      <c r="G52" s="19"/>
-      <c r="H52" s="19"/>
-      <c r="I52" s="19"/>
-      <c r="J52" s="19"/>
-      <c r="K52" s="19"/>
-      <c r="L52" s="19"/>
-      <c r="M52" s="19"/>
-      <c r="N52" s="19"/>
-      <c r="O52" s="19"/>
-      <c r="P52" s="19"/>
-      <c r="Q52" s="19"/>
-      <c r="R52" s="19"/>
-      <c r="S52" s="19"/>
-      <c r="T52" s="19"/>
-      <c r="U52" s="19"/>
-      <c r="V52" s="19"/>
-      <c r="W52" s="19"/>
-    </row>
-    <row r="53" spans="1:23" ht="26.45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="19" t="s">
+      <c r="B52" s="20"/>
+      <c r="C52" s="20"/>
+      <c r="D52" s="20"/>
+      <c r="E52" s="20"/>
+      <c r="F52" s="20"/>
+      <c r="G52" s="20"/>
+      <c r="H52" s="20"/>
+      <c r="I52" s="20"/>
+      <c r="J52" s="20"/>
+      <c r="K52" s="20"/>
+      <c r="L52" s="20"/>
+      <c r="M52" s="20"/>
+      <c r="N52" s="20"/>
+      <c r="O52" s="20"/>
+      <c r="P52" s="20"/>
+      <c r="Q52" s="20"/>
+      <c r="R52" s="20"/>
+      <c r="S52" s="20"/>
+      <c r="T52" s="20"/>
+      <c r="U52" s="20"/>
+      <c r="V52" s="20"/>
+      <c r="W52" s="20"/>
+      <c r="X52" s="20"/>
+    </row>
+    <row r="53" spans="1:24" ht="26.45" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A53" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="B53" s="19"/>
-      <c r="C53" s="19"/>
-      <c r="D53" s="19"/>
-      <c r="E53" s="19"/>
-      <c r="F53" s="19"/>
-      <c r="G53" s="19"/>
-      <c r="H53" s="19"/>
-      <c r="I53" s="19"/>
-      <c r="J53" s="19"/>
-      <c r="K53" s="19"/>
-      <c r="L53" s="19"/>
-      <c r="M53" s="19"/>
-      <c r="N53" s="19"/>
-      <c r="O53" s="19"/>
-      <c r="P53" s="19"/>
-      <c r="Q53" s="19"/>
-      <c r="R53" s="19"/>
-      <c r="S53" s="19"/>
-      <c r="T53" s="19"/>
-      <c r="U53" s="19"/>
-      <c r="V53" s="19"/>
-      <c r="W53" s="19"/>
-    </row>
-    <row r="54" spans="1:23" ht="40.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="19" t="s">
+      <c r="B53" s="20"/>
+      <c r="C53" s="20"/>
+      <c r="D53" s="20"/>
+      <c r="E53" s="20"/>
+      <c r="F53" s="20"/>
+      <c r="G53" s="20"/>
+      <c r="H53" s="20"/>
+      <c r="I53" s="20"/>
+      <c r="J53" s="20"/>
+      <c r="K53" s="20"/>
+      <c r="L53" s="20"/>
+      <c r="M53" s="20"/>
+      <c r="N53" s="20"/>
+      <c r="O53" s="20"/>
+      <c r="P53" s="20"/>
+      <c r="Q53" s="20"/>
+      <c r="R53" s="20"/>
+      <c r="S53" s="20"/>
+      <c r="T53" s="20"/>
+      <c r="U53" s="20"/>
+      <c r="V53" s="20"/>
+      <c r="W53" s="20"/>
+      <c r="X53" s="20"/>
+    </row>
+    <row r="54" spans="1:24" ht="40.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A54" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="B54" s="19"/>
-      <c r="C54" s="19"/>
-      <c r="D54" s="19"/>
-      <c r="E54" s="19"/>
-      <c r="F54" s="19"/>
-      <c r="G54" s="19"/>
-      <c r="H54" s="19"/>
-      <c r="I54" s="19"/>
-      <c r="J54" s="19"/>
-      <c r="K54" s="19"/>
-      <c r="L54" s="19"/>
-      <c r="M54" s="19"/>
-      <c r="N54" s="19"/>
-      <c r="O54" s="19"/>
-      <c r="P54" s="19"/>
-      <c r="Q54" s="19"/>
-      <c r="R54" s="19"/>
-      <c r="S54" s="19"/>
-      <c r="T54" s="19"/>
-      <c r="U54" s="19"/>
-      <c r="V54" s="19"/>
-      <c r="W54" s="19"/>
-    </row>
-    <row r="55" spans="1:23" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="19" t="s">
+      <c r="B54" s="20"/>
+      <c r="C54" s="20"/>
+      <c r="D54" s="20"/>
+      <c r="E54" s="20"/>
+      <c r="F54" s="20"/>
+      <c r="G54" s="20"/>
+      <c r="H54" s="20"/>
+      <c r="I54" s="20"/>
+      <c r="J54" s="20"/>
+      <c r="K54" s="20"/>
+      <c r="L54" s="20"/>
+      <c r="M54" s="20"/>
+      <c r="N54" s="20"/>
+      <c r="O54" s="20"/>
+      <c r="P54" s="20"/>
+      <c r="Q54" s="20"/>
+      <c r="R54" s="20"/>
+      <c r="S54" s="20"/>
+      <c r="T54" s="20"/>
+      <c r="U54" s="20"/>
+      <c r="V54" s="20"/>
+      <c r="W54" s="20"/>
+      <c r="X54" s="20"/>
+    </row>
+    <row r="55" spans="1:24" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A55" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="B55" s="20"/>
-      <c r="C55" s="20"/>
-      <c r="D55" s="20"/>
-      <c r="E55" s="20"/>
-      <c r="F55" s="20"/>
-      <c r="G55" s="20"/>
-      <c r="H55" s="20"/>
-      <c r="I55" s="20"/>
-      <c r="J55" s="20"/>
-      <c r="K55" s="20"/>
-      <c r="L55" s="20"/>
-      <c r="M55" s="20"/>
-      <c r="N55" s="20"/>
-      <c r="O55" s="20"/>
-      <c r="P55" s="20"/>
-      <c r="Q55" s="20"/>
-      <c r="R55" s="20"/>
-      <c r="S55" s="20"/>
-      <c r="T55" s="20"/>
-      <c r="U55" s="20"/>
-      <c r="V55" s="20"/>
-      <c r="W55" s="20"/>
-    </row>
-    <row r="56" spans="1:23" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="19" t="s">
+      <c r="B55" s="23"/>
+      <c r="C55" s="23"/>
+      <c r="D55" s="23"/>
+      <c r="E55" s="23"/>
+      <c r="F55" s="23"/>
+      <c r="G55" s="23"/>
+      <c r="H55" s="23"/>
+      <c r="I55" s="23"/>
+      <c r="J55" s="23"/>
+      <c r="K55" s="23"/>
+      <c r="L55" s="23"/>
+      <c r="M55" s="23"/>
+      <c r="N55" s="23"/>
+      <c r="O55" s="23"/>
+      <c r="P55" s="23"/>
+      <c r="Q55" s="23"/>
+      <c r="R55" s="23"/>
+      <c r="S55" s="23"/>
+      <c r="T55" s="23"/>
+      <c r="U55" s="23"/>
+      <c r="V55" s="23"/>
+      <c r="W55" s="23"/>
+      <c r="X55" s="23"/>
+    </row>
+    <row r="56" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A56" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="B56" s="19"/>
-      <c r="C56" s="19"/>
-      <c r="D56" s="19"/>
-      <c r="E56" s="19"/>
-      <c r="F56" s="19"/>
-      <c r="G56" s="19"/>
-      <c r="H56" s="19"/>
-      <c r="I56" s="19"/>
-      <c r="J56" s="19"/>
-      <c r="K56" s="19"/>
-      <c r="L56" s="19"/>
-      <c r="M56" s="19"/>
-      <c r="N56" s="19"/>
-      <c r="O56" s="19"/>
-      <c r="P56" s="19"/>
-      <c r="Q56" s="19"/>
-      <c r="R56" s="19"/>
-      <c r="S56" s="19"/>
-      <c r="T56" s="19"/>
-      <c r="U56" s="19"/>
-      <c r="V56" s="19"/>
-      <c r="W56" s="19"/>
-    </row>
-    <row r="57" spans="1:23" ht="78" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A57" s="19" t="s">
+      <c r="B56" s="20"/>
+      <c r="C56" s="20"/>
+      <c r="D56" s="20"/>
+      <c r="E56" s="20"/>
+      <c r="F56" s="20"/>
+      <c r="G56" s="20"/>
+      <c r="H56" s="20"/>
+      <c r="I56" s="20"/>
+      <c r="J56" s="20"/>
+      <c r="K56" s="20"/>
+      <c r="L56" s="20"/>
+      <c r="M56" s="20"/>
+      <c r="N56" s="20"/>
+      <c r="O56" s="20"/>
+      <c r="P56" s="20"/>
+      <c r="Q56" s="20"/>
+      <c r="R56" s="20"/>
+      <c r="S56" s="20"/>
+      <c r="T56" s="20"/>
+      <c r="U56" s="20"/>
+      <c r="V56" s="20"/>
+      <c r="W56" s="20"/>
+      <c r="X56" s="20"/>
+    </row>
+    <row r="57" spans="1:24" ht="78" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A57" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="B57" s="19"/>
-      <c r="C57" s="19"/>
-      <c r="D57" s="19"/>
-      <c r="E57" s="19"/>
-      <c r="F57" s="19"/>
-      <c r="G57" s="19"/>
-      <c r="H57" s="19"/>
-      <c r="I57" s="19"/>
-      <c r="J57" s="19"/>
-      <c r="K57" s="19"/>
-      <c r="L57" s="19"/>
-      <c r="M57" s="19"/>
-      <c r="N57" s="19"/>
-      <c r="O57" s="19"/>
-      <c r="P57" s="19"/>
-      <c r="Q57" s="19"/>
-      <c r="R57" s="19"/>
-      <c r="S57" s="19"/>
-      <c r="T57" s="19"/>
-      <c r="U57" s="19"/>
-      <c r="V57" s="19"/>
-      <c r="W57" s="19"/>
-    </row>
-    <row r="58" spans="1:23" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A58" s="21" t="s">
+      <c r="B57" s="20"/>
+      <c r="C57" s="20"/>
+      <c r="D57" s="20"/>
+      <c r="E57" s="20"/>
+      <c r="F57" s="20"/>
+      <c r="G57" s="20"/>
+      <c r="H57" s="20"/>
+      <c r="I57" s="20"/>
+      <c r="J57" s="20"/>
+      <c r="K57" s="20"/>
+      <c r="L57" s="20"/>
+      <c r="M57" s="20"/>
+      <c r="N57" s="20"/>
+      <c r="O57" s="20"/>
+      <c r="P57" s="20"/>
+      <c r="Q57" s="20"/>
+      <c r="R57" s="20"/>
+      <c r="S57" s="20"/>
+      <c r="T57" s="20"/>
+      <c r="U57" s="20"/>
+      <c r="V57" s="20"/>
+      <c r="W57" s="20"/>
+      <c r="X57" s="20"/>
+    </row>
+    <row r="58" spans="1:24" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A58" s="26" t="s">
         <v>88</v>
       </c>
-      <c r="B58" s="21"/>
-      <c r="C58" s="21"/>
-      <c r="D58" s="21"/>
-      <c r="E58" s="21"/>
-      <c r="F58" s="21"/>
-      <c r="G58" s="21"/>
-      <c r="H58" s="21"/>
-      <c r="I58" s="21"/>
-      <c r="J58" s="21"/>
-      <c r="K58" s="21"/>
-      <c r="L58" s="21"/>
-      <c r="M58" s="21"/>
-      <c r="N58" s="21"/>
-      <c r="O58" s="21"/>
-      <c r="P58" s="21"/>
-      <c r="Q58" s="21"/>
-      <c r="R58" s="21"/>
-      <c r="S58" s="21"/>
-      <c r="T58" s="21"/>
-      <c r="U58" s="21"/>
-      <c r="V58" s="21"/>
-      <c r="W58" s="21"/>
-    </row>
-    <row r="59" spans="1:23" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A59" s="19" t="s">
+      <c r="B58" s="26"/>
+      <c r="C58" s="26"/>
+      <c r="D58" s="26"/>
+      <c r="E58" s="26"/>
+      <c r="F58" s="26"/>
+      <c r="G58" s="26"/>
+      <c r="H58" s="26"/>
+      <c r="I58" s="26"/>
+      <c r="J58" s="26"/>
+      <c r="K58" s="26"/>
+      <c r="L58" s="26"/>
+      <c r="M58" s="26"/>
+      <c r="N58" s="26"/>
+      <c r="O58" s="26"/>
+      <c r="P58" s="26"/>
+      <c r="Q58" s="26"/>
+      <c r="R58" s="26"/>
+      <c r="S58" s="26"/>
+      <c r="T58" s="26"/>
+      <c r="U58" s="26"/>
+      <c r="V58" s="26"/>
+      <c r="W58" s="26"/>
+      <c r="X58" s="26"/>
+    </row>
+    <row r="59" spans="1:24" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A59" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="B59" s="19"/>
-      <c r="C59" s="19"/>
-      <c r="D59" s="19"/>
-      <c r="E59" s="19"/>
-      <c r="F59" s="19"/>
-      <c r="G59" s="19"/>
-      <c r="H59" s="19"/>
-      <c r="I59" s="19"/>
-      <c r="J59" s="19"/>
-      <c r="K59" s="19"/>
-      <c r="L59" s="19"/>
-      <c r="M59" s="19"/>
-      <c r="N59" s="19"/>
-      <c r="O59" s="19"/>
-      <c r="P59" s="19"/>
-      <c r="Q59" s="19"/>
-      <c r="R59" s="19"/>
-      <c r="S59" s="19"/>
-      <c r="T59" s="19"/>
-      <c r="U59" s="19"/>
-      <c r="V59" s="19"/>
-      <c r="W59" s="19"/>
-    </row>
-    <row r="60" spans="1:23" ht="39" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A60" s="19" t="s">
+      <c r="B59" s="20"/>
+      <c r="C59" s="20"/>
+      <c r="D59" s="20"/>
+      <c r="E59" s="20"/>
+      <c r="F59" s="20"/>
+      <c r="G59" s="20"/>
+      <c r="H59" s="20"/>
+      <c r="I59" s="20"/>
+      <c r="J59" s="20"/>
+      <c r="K59" s="20"/>
+      <c r="L59" s="20"/>
+      <c r="M59" s="20"/>
+      <c r="N59" s="20"/>
+      <c r="O59" s="20"/>
+      <c r="P59" s="20"/>
+      <c r="Q59" s="20"/>
+      <c r="R59" s="20"/>
+      <c r="S59" s="20"/>
+      <c r="T59" s="20"/>
+      <c r="U59" s="20"/>
+      <c r="V59" s="20"/>
+      <c r="W59" s="20"/>
+      <c r="X59" s="20"/>
+    </row>
+    <row r="60" spans="1:24" ht="39" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A60" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="B60" s="19"/>
-      <c r="C60" s="19"/>
-      <c r="D60" s="19"/>
-      <c r="E60" s="19"/>
-      <c r="F60" s="19"/>
-      <c r="G60" s="19"/>
-      <c r="H60" s="19"/>
-      <c r="I60" s="19"/>
-      <c r="J60" s="19"/>
-      <c r="K60" s="19"/>
-      <c r="L60" s="19"/>
-      <c r="M60" s="19"/>
-      <c r="N60" s="19"/>
-      <c r="O60" s="19"/>
-      <c r="P60" s="19"/>
-      <c r="Q60" s="19"/>
-      <c r="R60" s="19"/>
-      <c r="S60" s="19"/>
-      <c r="T60" s="19"/>
-      <c r="U60" s="19"/>
-      <c r="V60" s="19"/>
-      <c r="W60" s="19"/>
-    </row>
-    <row r="61" spans="1:23" ht="80.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A61" s="19" t="s">
+      <c r="B60" s="20"/>
+      <c r="C60" s="20"/>
+      <c r="D60" s="20"/>
+      <c r="E60" s="20"/>
+      <c r="F60" s="20"/>
+      <c r="G60" s="20"/>
+      <c r="H60" s="20"/>
+      <c r="I60" s="20"/>
+      <c r="J60" s="20"/>
+      <c r="K60" s="20"/>
+      <c r="L60" s="20"/>
+      <c r="M60" s="20"/>
+      <c r="N60" s="20"/>
+      <c r="O60" s="20"/>
+      <c r="P60" s="20"/>
+      <c r="Q60" s="20"/>
+      <c r="R60" s="20"/>
+      <c r="S60" s="20"/>
+      <c r="T60" s="20"/>
+      <c r="U60" s="20"/>
+      <c r="V60" s="20"/>
+      <c r="W60" s="20"/>
+      <c r="X60" s="20"/>
+    </row>
+    <row r="61" spans="1:24" ht="80.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A61" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="B61" s="19"/>
-      <c r="C61" s="19"/>
-      <c r="D61" s="19"/>
-      <c r="E61" s="19"/>
-      <c r="F61" s="19"/>
-      <c r="G61" s="19"/>
-      <c r="H61" s="19"/>
-      <c r="I61" s="19"/>
-      <c r="J61" s="19"/>
-      <c r="K61" s="19"/>
-      <c r="L61" s="19"/>
-      <c r="M61" s="19"/>
-      <c r="N61" s="19"/>
-      <c r="O61" s="19"/>
-      <c r="P61" s="19"/>
-      <c r="Q61" s="19"/>
-      <c r="R61" s="19"/>
-      <c r="S61" s="19"/>
-      <c r="T61" s="19"/>
-      <c r="U61" s="19"/>
-      <c r="V61" s="19"/>
-      <c r="W61" s="19"/>
-    </row>
-    <row r="62" spans="1:23" ht="86.1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A62" s="19" t="s">
+      <c r="B61" s="20"/>
+      <c r="C61" s="20"/>
+      <c r="D61" s="20"/>
+      <c r="E61" s="20"/>
+      <c r="F61" s="20"/>
+      <c r="G61" s="20"/>
+      <c r="H61" s="20"/>
+      <c r="I61" s="20"/>
+      <c r="J61" s="20"/>
+      <c r="K61" s="20"/>
+      <c r="L61" s="20"/>
+      <c r="M61" s="20"/>
+      <c r="N61" s="20"/>
+      <c r="O61" s="20"/>
+      <c r="P61" s="20"/>
+      <c r="Q61" s="20"/>
+      <c r="R61" s="20"/>
+      <c r="S61" s="20"/>
+      <c r="T61" s="20"/>
+      <c r="U61" s="20"/>
+      <c r="V61" s="20"/>
+      <c r="W61" s="20"/>
+      <c r="X61" s="20"/>
+    </row>
+    <row r="62" spans="1:24" ht="86.1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A62" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="B62" s="19"/>
-      <c r="C62" s="19"/>
-      <c r="D62" s="19"/>
-      <c r="E62" s="19"/>
-      <c r="F62" s="19"/>
-      <c r="G62" s="19"/>
-      <c r="H62" s="19"/>
-      <c r="I62" s="19"/>
-      <c r="J62" s="19"/>
-      <c r="K62" s="19"/>
-      <c r="L62" s="19"/>
-      <c r="M62" s="19"/>
-      <c r="N62" s="19"/>
-      <c r="O62" s="19"/>
-      <c r="P62" s="19"/>
-      <c r="Q62" s="19"/>
-      <c r="R62" s="19"/>
-      <c r="S62" s="19"/>
-      <c r="T62" s="19"/>
-      <c r="U62" s="19"/>
-      <c r="V62" s="19"/>
-      <c r="W62" s="19"/>
-    </row>
-    <row r="64" spans="1:23" ht="13.15" x14ac:dyDescent="0.4">
+      <c r="B62" s="20"/>
+      <c r="C62" s="20"/>
+      <c r="D62" s="20"/>
+      <c r="E62" s="20"/>
+      <c r="F62" s="20"/>
+      <c r="G62" s="20"/>
+      <c r="H62" s="20"/>
+      <c r="I62" s="20"/>
+      <c r="J62" s="20"/>
+      <c r="K62" s="20"/>
+      <c r="L62" s="20"/>
+      <c r="M62" s="20"/>
+      <c r="N62" s="20"/>
+      <c r="O62" s="20"/>
+      <c r="P62" s="20"/>
+      <c r="Q62" s="20"/>
+      <c r="R62" s="20"/>
+      <c r="S62" s="20"/>
+      <c r="T62" s="20"/>
+      <c r="U62" s="20"/>
+      <c r="V62" s="20"/>
+      <c r="W62" s="20"/>
+      <c r="X62" s="20"/>
+    </row>
+    <row r="64" spans="1:24" ht="13.15" x14ac:dyDescent="0.4">
       <c r="A64" t="s">
         <v>93</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="A53:W53"/>
-    <mergeCell ref="A49:W49"/>
-    <mergeCell ref="A52:W52"/>
-    <mergeCell ref="A1:W1"/>
+    <mergeCell ref="A62:X62"/>
+    <mergeCell ref="A60:X60"/>
+    <mergeCell ref="A61:X61"/>
+    <mergeCell ref="A54:X54"/>
+    <mergeCell ref="A56:X56"/>
+    <mergeCell ref="A57:X57"/>
+    <mergeCell ref="A59:X59"/>
+    <mergeCell ref="A55:X55"/>
+    <mergeCell ref="A58:X58"/>
+    <mergeCell ref="A53:X53"/>
+    <mergeCell ref="A49:X49"/>
+    <mergeCell ref="A52:X52"/>
+    <mergeCell ref="A1:X1"/>
     <mergeCell ref="A42:Q42"/>
     <mergeCell ref="A43:Q43"/>
     <mergeCell ref="A41:Q41"/>
     <mergeCell ref="A48:B48"/>
-    <mergeCell ref="A45:W45"/>
-    <mergeCell ref="A44:W44"/>
-    <mergeCell ref="A46:W46"/>
-    <mergeCell ref="A47:W47"/>
-    <mergeCell ref="A50:W50"/>
-    <mergeCell ref="A51:W51"/>
-    <mergeCell ref="A62:W62"/>
-    <mergeCell ref="A60:W60"/>
-    <mergeCell ref="A61:W61"/>
-    <mergeCell ref="A54:W54"/>
-    <mergeCell ref="A56:W56"/>
-    <mergeCell ref="A57:W57"/>
-    <mergeCell ref="A59:W59"/>
-    <mergeCell ref="A55:W55"/>
-    <mergeCell ref="A58:W58"/>
+    <mergeCell ref="A45:X45"/>
+    <mergeCell ref="A44:X44"/>
+    <mergeCell ref="A46:X46"/>
+    <mergeCell ref="A47:X47"/>
+    <mergeCell ref="A50:X50"/>
+    <mergeCell ref="A51:X51"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
vat_rate: source data updated
</commit_message>
<xml_diff>
--- a/source_data/oecd_vat_gst_rates_ctt_trends.xlsx
+++ b/source_data/oecd_vat_gst_rates_ctt_trends.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\international-tax-competitiveness-index\source_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexanderMengden\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27E2BE37-5B82-44E7-BF95-47BE14842A5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C145109-51D4-431D-ACC6-FC0F8A8C2C95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="99">
   <si>
     <t>Australia</t>
   </si>
@@ -75,52 +75,19 @@
     <t>* See country notes</t>
   </si>
   <si>
-    <t>10.0/13.0</t>
-  </si>
-  <si>
     <t>0.0/6.0/12.0</t>
   </si>
   <si>
     <t>-</t>
   </si>
   <si>
-    <t>13.0/15.0</t>
-  </si>
-  <si>
     <t>0.0/5.0</t>
   </si>
   <si>
-    <t>0.0/10.0/14.0</t>
-  </si>
-  <si>
-    <t>2.1/5.5/10.0</t>
-  </si>
-  <si>
-    <t>0.9/2.1/10.0/13.0 &amp; 1.05/1.75/2.1/8.5</t>
-  </si>
-  <si>
-    <t>6.0/13.0</t>
-  </si>
-  <si>
     <t>0.0/11.0</t>
   </si>
   <si>
     <t>0.0/4.8/9.0/13.5</t>
-  </si>
-  <si>
-    <t>4.0/5.0/10.0</t>
-  </si>
-  <si>
-    <t>5.0/9.0</t>
-  </si>
-  <si>
-    <t>3.0/8.0/14.0</t>
-  </si>
-  <si>
-    <t>5.0/8.0</t>
-  </si>
-  <si>
-    <t>5.0/9.5</t>
   </si>
   <si>
     <t>Austria*</t>
@@ -201,15 +168,9 @@
     <t>* Country notes:</t>
   </si>
   <si>
-    <t>7.0/0.0</t>
-  </si>
-  <si>
     <t>Belgium</t>
   </si>
   <si>
-    <t>1.0/10.0</t>
-  </si>
-  <si>
     <t>Estonia</t>
   </si>
   <si>
@@ -246,40 +207,13 @@
     <t xml:space="preserve"> - </t>
   </si>
   <si>
-    <t>0/12.0</t>
-  </si>
-  <si>
-    <t>0.0/9.0/13.0</t>
-  </si>
-  <si>
     <t>0/5.0/18.0</t>
   </si>
   <si>
-    <t>4.0/9.0/12.0/16.0/22.0</t>
-  </si>
-  <si>
-    <t>5.0/19</t>
-  </si>
-  <si>
     <t>0.0/2.6/3.8</t>
   </si>
   <si>
-    <t>0/4.0/10.0</t>
-  </si>
-  <si>
-    <t>0/4.0/6.0/13.0</t>
-  </si>
-  <si>
     <t>3.0/4.0/9.0/17.0</t>
-  </si>
-  <si>
-    <t>0/1.0/2.0/4.0</t>
-  </si>
-  <si>
-    <t>5.0/12.0</t>
-  </si>
-  <si>
-    <t>0.0/12.0/15.0</t>
   </si>
   <si>
     <t xml:space="preserve">0.0/0.5/1.0/3.0/4.0/5.0/6.0/7.0/8.0/9.0/ 
@@ -323,33 +257,6 @@
       </rPr>
       <t xml:space="preserve">*. A standard rate of 19% applies in Jungholz and Mittelberg. A specific temporary zero VAT 
 rate applies to the supply and installation of solar panels – See country note to Annex Table 2.A.2. </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Canada</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">. The following provinces have harmonised their provincial sales taxes with the federal Goods 
-and Services Tax and therefore levy a GST/HST at the following rates: New Brunswick, Newfoundland 
-and Labrador, Nova Scotia, Prince Edward Island: 15%; and Ontario: 13%. Québec applies GST at a 
-rate of 5% and Québec Sales Tax at a rate of 9.975% (applied on the same tax base as the GST). With 
-the exception of Canada’s territories (Yukon, Northwest Territories and Nunavut) and the province of 
-Alberta, other Canadian provinces apply a provincial sales tax to certain goods and services in addition 
-to the federal GST. </t>
     </r>
   </si>
   <si>
@@ -668,6 +575,132 @@
       <t>: Temporary VAT rate reductions are shown in italics in the country notes above.</t>
     </r>
   </si>
+  <si>
+    <t>(0.0)/10.0/13.0</t>
+  </si>
+  <si>
+    <t>0.0/9.0</t>
+  </si>
+  <si>
+    <t>0.9/10.0/13.0 &amp; 1.05/1.75/2.1/8.5</t>
+  </si>
+  <si>
+    <t>0.0/7.0</t>
+  </si>
+  <si>
+    <t>4.0/5.0/9.0/12.0/16.0/22.0</t>
+  </si>
+  <si>
+    <t>0.0</t>
+  </si>
+  <si>
+    <t>8.0</t>
+  </si>
+  <si>
+    <t>0.0/12.0</t>
+  </si>
+  <si>
+    <t>19.0</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Canada</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">. The following provinces have harmonised their provincial sales taxes with the federal Goods 
+and Services Tax and therefore levy a GST/HST at the following rates: New Brunswick, Newfoundland 
+and Labrador, Prince Edward Island: 15%; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Nova Scotia: 14% (1 April 2025);</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> and Ontario: 13%. Québec applies GST at a 
+rate of 5% and Québec Sales Tax at a rate of 9.975% (applied on the same tax base as the GST). With 
+the exception of Canada’s territories (Yukon, Northwest Territories and Nunavut) and the province of 
+Alberta, other Canadian provinces apply a provincial sales tax to certain goods and services in addition 
+to the federal GST. </t>
+    </r>
+  </si>
+  <si>
+    <t>0.0/4.0/6.0/13.0</t>
+  </si>
+  <si>
+    <t>0.0/4.0/5.0/10.0</t>
+  </si>
+  <si>
+    <t>0.0/5.0/12.0</t>
+  </si>
+  <si>
+    <t>0.0/5.0/8.0</t>
+  </si>
+  <si>
+    <t>0.0/6.0/13.0</t>
+  </si>
+  <si>
+    <t>0.0/4.0/10.0</t>
+  </si>
+  <si>
+    <t>0.0/1.0/10.0</t>
+  </si>
+  <si>
+    <t>13.0/14.0/15.0</t>
+  </si>
+  <si>
+    <t>0.0/0.5/1.0/2.0/4.0/10.0</t>
+  </si>
+  <si>
+    <t>0.0/9.0/13.0</t>
+  </si>
+  <si>
+    <t>0.0/10.0/13.5</t>
+  </si>
+  <si>
+    <t>0.0/2.1/5.5/10.0</t>
+  </si>
+  <si>
+    <t>0.0/8.0</t>
+  </si>
+  <si>
+    <t>0.0/5.0/9.0</t>
+  </si>
+  <si>
+    <t>0.0/3.0/8.0/14.0</t>
+  </si>
+  <si>
+    <t>0.0/11.11/12.0/15.0</t>
+  </si>
+  <si>
+    <t>0.0/5.0/19.0</t>
+  </si>
+  <si>
+    <t>0.0/5.0/9.5</t>
+  </si>
 </sst>
 </file>
 
@@ -676,7 +709,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -727,6 +760,17 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF00B0F0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8.5"/>
+      <name val="Arial Narrow"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -861,7 +905,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -895,9 +939,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
@@ -910,9 +951,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -935,6 +973,27 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -950,6 +1009,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1227,32 +1290,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="14.65" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="21" t="s">
-        <v>46</v>
-      </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="21"/>
-      <c r="O1" s="21"/>
-      <c r="P1" s="21"/>
-      <c r="Q1" s="21"/>
-      <c r="R1" s="21"/>
-      <c r="S1" s="21"/>
-      <c r="T1" s="21"/>
-      <c r="U1" s="21"/>
-      <c r="V1" s="21"/>
-      <c r="W1" s="21"/>
-      <c r="X1" s="21"/>
+      <c r="A1" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
+      <c r="O1" s="19"/>
+      <c r="P1" s="19"/>
+      <c r="Q1" s="19"/>
+      <c r="R1" s="19"/>
+      <c r="S1" s="19"/>
+      <c r="T1" s="19"/>
+      <c r="U1" s="19"/>
+      <c r="V1" s="19"/>
+      <c r="W1" s="19"/>
+      <c r="X1" s="19"/>
     </row>
     <row r="2" spans="1:24" ht="50.1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B2" s="12">
@@ -1318,10 +1381,10 @@
       <c r="V2" s="12">
         <v>2026</v>
       </c>
-      <c r="W2" s="18" t="s">
+      <c r="W2" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="X2" s="16" t="s">
+      <c r="X2" s="15" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1389,17 +1452,19 @@
       <c r="U3" s="9">
         <v>10</v>
       </c>
-      <c r="V3" s="9"/>
-      <c r="W3" s="13">
-        <v>0</v>
-      </c>
-      <c r="X3" s="13" t="s">
-        <v>12</v>
+      <c r="V3" s="9">
+        <v>10</v>
+      </c>
+      <c r="W3" s="28" t="s">
+        <v>76</v>
+      </c>
+      <c r="X3" s="28" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="B4" s="10">
         <v>20</v>
@@ -1461,17 +1526,19 @@
       <c r="U4" s="10">
         <v>20</v>
       </c>
-      <c r="V4" s="10"/>
-      <c r="W4" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="X4" s="14">
-        <v>19</v>
+      <c r="V4" s="10">
+        <v>20</v>
+      </c>
+      <c r="W4" s="29" t="s">
+        <v>71</v>
+      </c>
+      <c r="X4" s="29" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="B5" s="11">
         <v>21</v>
@@ -1533,17 +1600,19 @@
       <c r="U5" s="11">
         <v>21</v>
       </c>
-      <c r="V5" s="11"/>
-      <c r="W5" s="15" t="s">
+      <c r="V5" s="11">
+        <v>21</v>
+      </c>
+      <c r="W5" s="30" t="s">
+        <v>10</v>
+      </c>
+      <c r="X5" s="30" t="s">
         <v>11</v>
-      </c>
-      <c r="X5" s="15" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B6" s="10">
         <v>7</v>
@@ -1605,12 +1674,14 @@
       <c r="U6" s="10">
         <v>5</v>
       </c>
-      <c r="V6" s="10"/>
-      <c r="W6" s="14">
-        <v>0</v>
-      </c>
-      <c r="X6" s="14" t="s">
-        <v>13</v>
+      <c r="V6" s="10">
+        <v>5</v>
+      </c>
+      <c r="W6" s="29" t="s">
+        <v>76</v>
+      </c>
+      <c r="X6" s="29" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.35">
@@ -1677,17 +1748,17 @@
       <c r="U7" s="11">
         <v>19</v>
       </c>
-      <c r="V7" s="11"/>
-      <c r="W7" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="X7" s="15" t="s">
-        <v>12</v>
+      <c r="V7" s="11">
+        <v>19</v>
+      </c>
+      <c r="W7" s="30"/>
+      <c r="X7" s="30" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="B8" s="10">
         <v>16</v>
@@ -1749,42 +1820,44 @@
       <c r="U8" s="10">
         <v>19</v>
       </c>
-      <c r="V8" s="10"/>
-      <c r="W8" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="X8" s="14" t="s">
+      <c r="V8" s="10">
+        <v>19</v>
+      </c>
+      <c r="W8" s="29" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="X8" s="29" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24" ht="22.5" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="11" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="D9" s="11"/>
       <c r="E9" s="11" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="G9" s="11"/>
       <c r="H9" s="11" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="I9" s="11" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="J9" s="11"/>
       <c r="K9" s="11" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="L9" s="11" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="M9" s="11"/>
       <c r="N9" s="11"/>
@@ -1809,15 +1882,19 @@
       <c r="U9" s="11">
         <v>13</v>
       </c>
-      <c r="V9" s="11"/>
-      <c r="W9" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="X9" s="15"/>
+      <c r="V9" s="11">
+        <v>13</v>
+      </c>
+      <c r="W9" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="X9" s="30" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="10" spans="1:24" ht="15.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="B10" s="10">
         <v>19</v>
@@ -1879,17 +1956,19 @@
       <c r="U10" s="10">
         <v>21</v>
       </c>
-      <c r="V10" s="10"/>
-      <c r="W10" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="X10" s="14" t="s">
-        <v>12</v>
+      <c r="V10" s="10">
+        <v>21</v>
+      </c>
+      <c r="W10" s="29" t="s">
+        <v>78</v>
+      </c>
+      <c r="X10" s="29" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>54</v>
+        <v>41</v>
       </c>
       <c r="B11" s="11">
         <v>25</v>
@@ -1951,17 +2030,19 @@
       <c r="U11" s="11">
         <v>25</v>
       </c>
-      <c r="V11" s="11"/>
-      <c r="W11" s="15">
-        <v>0</v>
-      </c>
-      <c r="X11" s="15" t="s">
-        <v>12</v>
+      <c r="V11" s="11">
+        <v>25</v>
+      </c>
+      <c r="W11" s="30" t="s">
+        <v>76</v>
+      </c>
+      <c r="X11" s="30" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B12" s="10">
         <v>18</v>
@@ -2023,17 +2104,19 @@
       <c r="U12" s="10">
         <v>24</v>
       </c>
-      <c r="V12" s="10"/>
-      <c r="W12" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="X12" s="14" t="s">
-        <v>12</v>
+      <c r="V12" s="10">
+        <v>24</v>
+      </c>
+      <c r="W12" s="29" t="s">
+        <v>90</v>
+      </c>
+      <c r="X12" s="29" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="B13" s="11">
         <v>22</v>
@@ -2095,17 +2178,19 @@
       <c r="U13" s="11">
         <v>25.5</v>
       </c>
-      <c r="V13" s="11"/>
-      <c r="W13" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="X13" s="15" t="s">
-        <v>12</v>
+      <c r="V13" s="25">
+        <v>25.5</v>
+      </c>
+      <c r="W13" s="30" t="s">
+        <v>91</v>
+      </c>
+      <c r="X13" s="30" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="14" spans="1:24" ht="22.5" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="B14" s="10">
         <v>19.600000000000001</v>
@@ -2167,17 +2252,19 @@
       <c r="U14" s="10">
         <v>20</v>
       </c>
-      <c r="V14" s="10"/>
-      <c r="W14" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="X14" s="14" t="s">
-        <v>17</v>
+      <c r="V14" s="10">
+        <v>20</v>
+      </c>
+      <c r="W14" s="29" t="s">
+        <v>92</v>
+      </c>
+      <c r="X14" s="29" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="B15" s="11">
         <v>16</v>
@@ -2239,17 +2326,19 @@
       <c r="U15" s="11">
         <v>19</v>
       </c>
-      <c r="V15" s="11"/>
-      <c r="W15" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="X15" s="15" t="s">
-        <v>12</v>
+      <c r="V15" s="11">
+        <v>19</v>
+      </c>
+      <c r="W15" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="X15" s="30" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="B16" s="10">
         <v>18</v>
@@ -2311,17 +2400,19 @@
       <c r="U16" s="10">
         <v>24</v>
       </c>
-      <c r="V16" s="10"/>
-      <c r="W16" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="X16" s="14" t="s">
-        <v>71</v>
+      <c r="V16" s="10">
+        <v>24</v>
+      </c>
+      <c r="W16" s="29" t="s">
+        <v>81</v>
+      </c>
+      <c r="X16" s="29" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="B17" s="11">
         <v>25</v>
@@ -2383,12 +2474,14 @@
       <c r="U17" s="11">
         <v>27</v>
       </c>
-      <c r="V17" s="11"/>
-      <c r="W17" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="X17" s="15" t="s">
-        <v>12</v>
+      <c r="V17" s="11">
+        <v>27</v>
+      </c>
+      <c r="W17" s="30" t="s">
+        <v>50</v>
+      </c>
+      <c r="X17" s="30" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="18" spans="1:24" x14ac:dyDescent="0.35">
@@ -2455,17 +2548,19 @@
       <c r="U18" s="10">
         <v>24</v>
       </c>
-      <c r="V18" s="10"/>
-      <c r="W18" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="X18" s="14" t="s">
-        <v>12</v>
+      <c r="V18" s="10">
+        <v>24</v>
+      </c>
+      <c r="W18" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="X18" s="29" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="B19" s="11">
         <v>21</v>
@@ -2527,17 +2622,19 @@
       <c r="U19" s="11">
         <v>23</v>
       </c>
-      <c r="V19" s="11"/>
-      <c r="W19" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="X19" s="15" t="s">
-        <v>12</v>
+      <c r="V19" s="11">
+        <v>23</v>
+      </c>
+      <c r="W19" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="X19" s="30" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="20" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="B20" s="10">
         <v>17</v>
@@ -2599,17 +2696,19 @@
       <c r="U20" s="10">
         <v>18</v>
       </c>
-      <c r="V20" s="10"/>
-      <c r="W20" s="14">
-        <v>0</v>
-      </c>
-      <c r="X20" s="14">
-        <v>0</v>
+      <c r="V20" s="26">
+        <v>18</v>
+      </c>
+      <c r="W20" s="29" t="s">
+        <v>76</v>
+      </c>
+      <c r="X20" s="29" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="B21" s="11">
         <v>20</v>
@@ -2671,17 +2770,19 @@
       <c r="U21" s="11">
         <v>22</v>
       </c>
-      <c r="V21" s="11"/>
-      <c r="W21" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="X21" s="15" t="s">
-        <v>12</v>
+      <c r="V21" s="11">
+        <v>22</v>
+      </c>
+      <c r="W21" s="30" t="s">
+        <v>82</v>
+      </c>
+      <c r="X21" s="30" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="22" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B22" s="10">
         <v>5</v>
@@ -2743,12 +2844,14 @@
       <c r="U22" s="10">
         <v>10</v>
       </c>
-      <c r="V22" s="10"/>
-      <c r="W22" s="14">
-        <v>8</v>
-      </c>
-      <c r="X22" s="14" t="s">
-        <v>12</v>
+      <c r="V22" s="10">
+        <v>10</v>
+      </c>
+      <c r="W22" s="29" t="s">
+        <v>93</v>
+      </c>
+      <c r="X22" s="29" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="23" spans="1:24" x14ac:dyDescent="0.35">
@@ -2815,17 +2918,19 @@
       <c r="U23" s="11">
         <v>10</v>
       </c>
-      <c r="V23" s="11"/>
-      <c r="W23" s="15">
-        <v>0</v>
-      </c>
-      <c r="X23" s="15" t="s">
-        <v>12</v>
+      <c r="V23" s="11">
+        <v>10</v>
+      </c>
+      <c r="W23" s="30" t="s">
+        <v>76</v>
+      </c>
+      <c r="X23" s="30" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="24" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="B24" s="10">
         <v>18</v>
@@ -2887,17 +2992,19 @@
       <c r="U24" s="10">
         <v>21</v>
       </c>
-      <c r="V24" s="10"/>
-      <c r="W24" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="X24" s="14" t="s">
-        <v>12</v>
+      <c r="V24" s="10">
+        <v>21</v>
+      </c>
+      <c r="W24" s="26" t="s">
+        <v>83</v>
+      </c>
+      <c r="X24" s="29" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="25" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="B25" s="11">
         <v>18</v>
@@ -2959,17 +3066,19 @@
       <c r="U25" s="11">
         <v>21</v>
       </c>
-      <c r="V25" s="11"/>
-      <c r="W25" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="X25" s="15" t="s">
-        <v>12</v>
+      <c r="V25" s="11">
+        <v>21</v>
+      </c>
+      <c r="W25" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="X25" s="30" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="26" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="B26" s="10">
         <v>15</v>
@@ -3031,17 +3140,19 @@
       <c r="U26" s="10">
         <v>17</v>
       </c>
-      <c r="V26" s="10"/>
-      <c r="W26" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="X26" s="14" t="s">
-        <v>12</v>
+      <c r="V26" s="10">
+        <v>17</v>
+      </c>
+      <c r="W26" s="29" t="s">
+        <v>95</v>
+      </c>
+      <c r="X26" s="29" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="27" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="B27" s="11">
         <v>15</v>
@@ -3103,17 +3214,19 @@
       <c r="U27" s="11">
         <v>16</v>
       </c>
-      <c r="V27" s="11"/>
-      <c r="W27" s="15">
-        <v>0</v>
-      </c>
-      <c r="X27" s="15">
-        <v>8</v>
+      <c r="V27" s="11">
+        <v>16</v>
+      </c>
+      <c r="W27" s="30" t="s">
+        <v>76</v>
+      </c>
+      <c r="X27" s="30" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="28" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="B28" s="10">
         <v>19</v>
@@ -3175,12 +3288,14 @@
       <c r="U28" s="10">
         <v>21</v>
       </c>
-      <c r="V28" s="10"/>
-      <c r="W28" s="14">
-        <v>9</v>
-      </c>
-      <c r="X28" s="14" t="s">
-        <v>12</v>
+      <c r="V28" s="10">
+        <v>21</v>
+      </c>
+      <c r="W28" s="29" t="s">
+        <v>72</v>
+      </c>
+      <c r="X28" s="29" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="29" spans="1:24" x14ac:dyDescent="0.35">
@@ -3247,17 +3362,19 @@
       <c r="U29" s="11">
         <v>15</v>
       </c>
-      <c r="V29" s="11"/>
-      <c r="W29" s="15">
-        <v>0</v>
-      </c>
-      <c r="X29" s="15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="V29" s="11">
+        <v>15</v>
+      </c>
+      <c r="W29" s="30" t="s">
+        <v>72</v>
+      </c>
+      <c r="X29" s="30" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="30" spans="1:24" ht="22.5" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="B30" s="10">
         <v>25</v>
@@ -3319,17 +3436,19 @@
       <c r="U30" s="10">
         <v>25</v>
       </c>
-      <c r="V30" s="10"/>
-      <c r="W30" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="X30" s="14" t="s">
-        <v>12</v>
+      <c r="V30" s="10">
+        <v>25</v>
+      </c>
+      <c r="W30" s="26" t="s">
+        <v>96</v>
+      </c>
+      <c r="X30" s="29" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="31" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="B31" s="11">
         <v>22</v>
@@ -3391,17 +3510,19 @@
       <c r="U31" s="11">
         <v>23</v>
       </c>
-      <c r="V31" s="11"/>
-      <c r="W31" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="X31" s="15" t="s">
-        <v>12</v>
+      <c r="V31" s="11">
+        <v>23</v>
+      </c>
+      <c r="W31" s="30" t="s">
+        <v>84</v>
+      </c>
+      <c r="X31" s="30" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="32" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="B32" s="10">
         <v>19</v>
@@ -3463,17 +3584,19 @@
       <c r="U32" s="10">
         <v>23</v>
       </c>
-      <c r="V32" s="10"/>
-      <c r="W32" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="X32" s="14" t="s">
-        <v>66</v>
+      <c r="V32" s="10">
+        <v>23</v>
+      </c>
+      <c r="W32" s="29" t="s">
+        <v>85</v>
+      </c>
+      <c r="X32" s="29" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="33" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="B33" s="11">
         <v>19</v>
@@ -3535,17 +3658,19 @@
       <c r="U33" s="11">
         <v>23</v>
       </c>
-      <c r="V33" s="11"/>
-      <c r="W33" s="19" t="s">
-        <v>67</v>
-      </c>
-      <c r="X33" s="15" t="s">
-        <v>12</v>
+      <c r="V33" s="27">
+        <v>23</v>
+      </c>
+      <c r="W33" s="31" t="s">
+        <v>97</v>
+      </c>
+      <c r="X33" s="30" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="34" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B34" s="10">
         <v>20</v>
@@ -3607,17 +3732,19 @@
       <c r="U34" s="10">
         <v>22</v>
       </c>
-      <c r="V34" s="10"/>
-      <c r="W34" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="X34" s="14" t="s">
-        <v>12</v>
+      <c r="V34" s="10">
+        <v>22</v>
+      </c>
+      <c r="W34" s="29" t="s">
+        <v>98</v>
+      </c>
+      <c r="X34" s="29" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="35" spans="1:24" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="B35" s="11">
         <v>16</v>
@@ -3679,17 +3806,19 @@
       <c r="U35" s="11">
         <v>21</v>
       </c>
-      <c r="V35" s="11"/>
-      <c r="W35" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="X35" s="15" t="s">
-        <v>75</v>
+      <c r="V35" s="11">
+        <v>21</v>
+      </c>
+      <c r="W35" s="30" t="s">
+        <v>86</v>
+      </c>
+      <c r="X35" s="30" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="36" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="B36" s="10">
         <v>25</v>
@@ -3751,17 +3880,19 @@
       <c r="U36" s="10">
         <v>25</v>
       </c>
-      <c r="V36" s="10"/>
-      <c r="W36" s="14" t="s">
+      <c r="V36" s="10">
+        <v>25</v>
+      </c>
+      <c r="W36" s="29" t="s">
+        <v>10</v>
+      </c>
+      <c r="X36" s="29" t="s">
         <v>11</v>
-      </c>
-      <c r="X36" s="14" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="37" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="B37" s="11">
         <v>7.6</v>
@@ -3823,17 +3954,19 @@
       <c r="U37" s="11">
         <v>8.1</v>
       </c>
-      <c r="V37" s="11"/>
-      <c r="W37" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="X37" s="15" t="s">
-        <v>12</v>
+      <c r="V37" s="11">
+        <v>8.1</v>
+      </c>
+      <c r="W37" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="X37" s="30" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="38" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="B38" s="10">
         <v>18</v>
@@ -3895,17 +4028,19 @@
       <c r="U38" s="10">
         <v>20</v>
       </c>
-      <c r="V38" s="10"/>
-      <c r="W38" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="X38" s="14" t="s">
-        <v>12</v>
+      <c r="V38" s="10">
+        <v>20</v>
+      </c>
+      <c r="W38" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="X38" s="13" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="39" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="B39" s="11">
         <v>17.5</v>
@@ -3967,12 +4102,14 @@
       <c r="U39" s="11">
         <v>20</v>
       </c>
-      <c r="V39" s="11"/>
-      <c r="W39" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="X39" s="15" t="s">
+      <c r="V39" s="11">
+        <v>20</v>
+      </c>
+      <c r="W39" s="14" t="s">
         <v>12</v>
+      </c>
+      <c r="X39" s="14" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="40" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4052,30 +4189,33 @@
         <f>AVERAGE(U3:U39)</f>
         <v>19.475675675675678</v>
       </c>
-      <c r="V40" s="7"/>
+      <c r="V40" s="7">
+        <f>AVERAGE(V3:V39)</f>
+        <v>19.475675675675678</v>
+      </c>
       <c r="W40" s="8"/>
-      <c r="X40" s="17"/>
+      <c r="X40" s="16"/>
     </row>
     <row r="41" spans="1:24" ht="17.45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="B41" s="25"/>
-      <c r="C41" s="25"/>
-      <c r="D41" s="25"/>
-      <c r="E41" s="25"/>
-      <c r="F41" s="25"/>
-      <c r="G41" s="25"/>
-      <c r="H41" s="25"/>
-      <c r="I41" s="25"/>
-      <c r="J41" s="25"/>
-      <c r="K41" s="25"/>
-      <c r="L41" s="25"/>
-      <c r="M41" s="25"/>
-      <c r="N41" s="25"/>
-      <c r="O41" s="25"/>
-      <c r="P41" s="25"/>
-      <c r="Q41" s="25"/>
+      <c r="A41" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="B41" s="23"/>
+      <c r="C41" s="23"/>
+      <c r="D41" s="23"/>
+      <c r="E41" s="23"/>
+      <c r="F41" s="23"/>
+      <c r="G41" s="23"/>
+      <c r="H41" s="23"/>
+      <c r="I41" s="23"/>
+      <c r="J41" s="23"/>
+      <c r="K41" s="23"/>
+      <c r="L41" s="23"/>
+      <c r="M41" s="23"/>
+      <c r="N41" s="23"/>
+      <c r="O41" s="23"/>
+      <c r="P41" s="23"/>
+      <c r="Q41" s="23"/>
       <c r="R41" s="3"/>
       <c r="S41" s="3"/>
       <c r="T41" s="3"/>
@@ -4083,25 +4223,25 @@
       <c r="V41" s="3"/>
     </row>
     <row r="42" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="A42" s="22" t="s">
+      <c r="A42" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="B42" s="23"/>
-      <c r="C42" s="23"/>
-      <c r="D42" s="23"/>
-      <c r="E42" s="23"/>
-      <c r="F42" s="23"/>
-      <c r="G42" s="23"/>
-      <c r="H42" s="23"/>
-      <c r="I42" s="23"/>
-      <c r="J42" s="23"/>
-      <c r="K42" s="23"/>
-      <c r="L42" s="23"/>
-      <c r="M42" s="23"/>
-      <c r="N42" s="23"/>
-      <c r="O42" s="23"/>
-      <c r="P42" s="23"/>
-      <c r="Q42" s="23"/>
+      <c r="B42" s="21"/>
+      <c r="C42" s="21"/>
+      <c r="D42" s="21"/>
+      <c r="E42" s="21"/>
+      <c r="F42" s="21"/>
+      <c r="G42" s="21"/>
+      <c r="H42" s="21"/>
+      <c r="I42" s="21"/>
+      <c r="J42" s="21"/>
+      <c r="K42" s="21"/>
+      <c r="L42" s="21"/>
+      <c r="M42" s="21"/>
+      <c r="N42" s="21"/>
+      <c r="O42" s="21"/>
+      <c r="P42" s="21"/>
+      <c r="Q42" s="21"/>
       <c r="R42" s="4"/>
       <c r="S42" s="4"/>
       <c r="T42" s="4"/>
@@ -4109,25 +4249,25 @@
       <c r="V42" s="4"/>
     </row>
     <row r="43" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="A43" s="23" t="s">
+      <c r="A43" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="B43" s="24"/>
-      <c r="C43" s="24"/>
-      <c r="D43" s="24"/>
-      <c r="E43" s="24"/>
-      <c r="F43" s="24"/>
-      <c r="G43" s="24"/>
-      <c r="H43" s="24"/>
-      <c r="I43" s="24"/>
-      <c r="J43" s="24"/>
-      <c r="K43" s="24"/>
-      <c r="L43" s="24"/>
-      <c r="M43" s="24"/>
-      <c r="N43" s="24"/>
-      <c r="O43" s="24"/>
-      <c r="P43" s="24"/>
-      <c r="Q43" s="24"/>
+      <c r="B43" s="22"/>
+      <c r="C43" s="22"/>
+      <c r="D43" s="22"/>
+      <c r="E43" s="22"/>
+      <c r="F43" s="22"/>
+      <c r="G43" s="22"/>
+      <c r="H43" s="22"/>
+      <c r="I43" s="22"/>
+      <c r="J43" s="22"/>
+      <c r="K43" s="22"/>
+      <c r="L43" s="22"/>
+      <c r="M43" s="22"/>
+      <c r="N43" s="22"/>
+      <c r="O43" s="22"/>
+      <c r="P43" s="22"/>
+      <c r="Q43" s="22"/>
       <c r="R43" s="5"/>
       <c r="S43" s="5"/>
       <c r="T43" s="5"/>
@@ -4135,515 +4275,515 @@
       <c r="V43" s="5"/>
     </row>
     <row r="44" spans="1:24" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="20" t="s">
-        <v>77</v>
-      </c>
-      <c r="B44" s="20"/>
-      <c r="C44" s="20"/>
-      <c r="D44" s="20"/>
-      <c r="E44" s="20"/>
-      <c r="F44" s="20"/>
-      <c r="G44" s="20"/>
-      <c r="H44" s="20"/>
-      <c r="I44" s="20"/>
-      <c r="J44" s="20"/>
-      <c r="K44" s="20"/>
-      <c r="L44" s="20"/>
-      <c r="M44" s="20"/>
-      <c r="N44" s="20"/>
-      <c r="O44" s="20"/>
-      <c r="P44" s="20"/>
-      <c r="Q44" s="20"/>
-      <c r="R44" s="20"/>
-      <c r="S44" s="20"/>
-      <c r="T44" s="20"/>
-      <c r="U44" s="20"/>
-      <c r="V44" s="20"/>
-      <c r="W44" s="20"/>
-      <c r="X44" s="20"/>
+      <c r="A44" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="B44" s="18"/>
+      <c r="C44" s="18"/>
+      <c r="D44" s="18"/>
+      <c r="E44" s="18"/>
+      <c r="F44" s="18"/>
+      <c r="G44" s="18"/>
+      <c r="H44" s="18"/>
+      <c r="I44" s="18"/>
+      <c r="J44" s="18"/>
+      <c r="K44" s="18"/>
+      <c r="L44" s="18"/>
+      <c r="M44" s="18"/>
+      <c r="N44" s="18"/>
+      <c r="O44" s="18"/>
+      <c r="P44" s="18"/>
+      <c r="Q44" s="18"/>
+      <c r="R44" s="18"/>
+      <c r="S44" s="18"/>
+      <c r="T44" s="18"/>
+      <c r="U44" s="18"/>
+      <c r="V44" s="18"/>
+      <c r="W44" s="18"/>
+      <c r="X44" s="18"/>
     </row>
     <row r="45" spans="1:24" ht="53.45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="20" t="s">
-        <v>78</v>
-      </c>
-      <c r="B45" s="20"/>
-      <c r="C45" s="20"/>
-      <c r="D45" s="20"/>
-      <c r="E45" s="20"/>
-      <c r="F45" s="20"/>
-      <c r="G45" s="20"/>
-      <c r="H45" s="20"/>
-      <c r="I45" s="20"/>
-      <c r="J45" s="20"/>
-      <c r="K45" s="20"/>
-      <c r="L45" s="20"/>
-      <c r="M45" s="20"/>
-      <c r="N45" s="20"/>
-      <c r="O45" s="20"/>
-      <c r="P45" s="20"/>
-      <c r="Q45" s="20"/>
-      <c r="R45" s="20"/>
-      <c r="S45" s="20"/>
-      <c r="T45" s="20"/>
-      <c r="U45" s="20"/>
-      <c r="V45" s="20"/>
-      <c r="W45" s="20"/>
-      <c r="X45" s="20"/>
+      <c r="A45" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="B45" s="18"/>
+      <c r="C45" s="18"/>
+      <c r="D45" s="18"/>
+      <c r="E45" s="18"/>
+      <c r="F45" s="18"/>
+      <c r="G45" s="18"/>
+      <c r="H45" s="18"/>
+      <c r="I45" s="18"/>
+      <c r="J45" s="18"/>
+      <c r="K45" s="18"/>
+      <c r="L45" s="18"/>
+      <c r="M45" s="18"/>
+      <c r="N45" s="18"/>
+      <c r="O45" s="18"/>
+      <c r="P45" s="18"/>
+      <c r="Q45" s="18"/>
+      <c r="R45" s="18"/>
+      <c r="S45" s="18"/>
+      <c r="T45" s="18"/>
+      <c r="U45" s="18"/>
+      <c r="V45" s="18"/>
+      <c r="W45" s="18"/>
+      <c r="X45" s="18"/>
     </row>
     <row r="46" spans="1:24" ht="15.6" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="20"/>
-      <c r="B46" s="20"/>
-      <c r="C46" s="20"/>
-      <c r="D46" s="20"/>
-      <c r="E46" s="20"/>
-      <c r="F46" s="20"/>
-      <c r="G46" s="20"/>
-      <c r="H46" s="20"/>
-      <c r="I46" s="20"/>
-      <c r="J46" s="20"/>
-      <c r="K46" s="20"/>
-      <c r="L46" s="20"/>
-      <c r="M46" s="20"/>
-      <c r="N46" s="20"/>
-      <c r="O46" s="20"/>
-      <c r="P46" s="20"/>
-      <c r="Q46" s="20"/>
-      <c r="R46" s="20"/>
-      <c r="S46" s="20"/>
-      <c r="T46" s="20"/>
-      <c r="U46" s="20"/>
-      <c r="V46" s="20"/>
-      <c r="W46" s="20"/>
-      <c r="X46" s="20"/>
+      <c r="A46" s="18"/>
+      <c r="B46" s="18"/>
+      <c r="C46" s="18"/>
+      <c r="D46" s="18"/>
+      <c r="E46" s="18"/>
+      <c r="F46" s="18"/>
+      <c r="G46" s="18"/>
+      <c r="H46" s="18"/>
+      <c r="I46" s="18"/>
+      <c r="J46" s="18"/>
+      <c r="K46" s="18"/>
+      <c r="L46" s="18"/>
+      <c r="M46" s="18"/>
+      <c r="N46" s="18"/>
+      <c r="O46" s="18"/>
+      <c r="P46" s="18"/>
+      <c r="Q46" s="18"/>
+      <c r="R46" s="18"/>
+      <c r="S46" s="18"/>
+      <c r="T46" s="18"/>
+      <c r="U46" s="18"/>
+      <c r="V46" s="18"/>
+      <c r="W46" s="18"/>
+      <c r="X46" s="18"/>
     </row>
     <row r="47" spans="1:24" ht="15.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="20"/>
-      <c r="B47" s="20"/>
-      <c r="C47" s="20"/>
-      <c r="D47" s="20"/>
-      <c r="E47" s="20"/>
-      <c r="F47" s="20"/>
-      <c r="G47" s="20"/>
-      <c r="H47" s="20"/>
-      <c r="I47" s="20"/>
-      <c r="J47" s="20"/>
-      <c r="K47" s="20"/>
-      <c r="L47" s="20"/>
-      <c r="M47" s="20"/>
-      <c r="N47" s="20"/>
-      <c r="O47" s="20"/>
-      <c r="P47" s="20"/>
-      <c r="Q47" s="20"/>
-      <c r="R47" s="20"/>
-      <c r="S47" s="20"/>
-      <c r="T47" s="20"/>
-      <c r="U47" s="20"/>
-      <c r="V47" s="20"/>
-      <c r="W47" s="20"/>
-      <c r="X47" s="20"/>
+      <c r="A47" s="18"/>
+      <c r="B47" s="18"/>
+      <c r="C47" s="18"/>
+      <c r="D47" s="18"/>
+      <c r="E47" s="18"/>
+      <c r="F47" s="18"/>
+      <c r="G47" s="18"/>
+      <c r="H47" s="18"/>
+      <c r="I47" s="18"/>
+      <c r="J47" s="18"/>
+      <c r="K47" s="18"/>
+      <c r="L47" s="18"/>
+      <c r="M47" s="18"/>
+      <c r="N47" s="18"/>
+      <c r="O47" s="18"/>
+      <c r="P47" s="18"/>
+      <c r="Q47" s="18"/>
+      <c r="R47" s="18"/>
+      <c r="S47" s="18"/>
+      <c r="T47" s="18"/>
+      <c r="U47" s="18"/>
+      <c r="V47" s="18"/>
+      <c r="W47" s="18"/>
+      <c r="X47" s="18"/>
     </row>
     <row r="48" spans="1:24" x14ac:dyDescent="0.35">
-      <c r="A48" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="B48" s="23"/>
+      <c r="A48" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B48" s="21"/>
       <c r="C48" s="4"/>
     </row>
     <row r="49" spans="1:24" ht="24.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="20" t="s">
-        <v>79</v>
-      </c>
-      <c r="B49" s="20"/>
-      <c r="C49" s="20"/>
-      <c r="D49" s="20"/>
-      <c r="E49" s="20"/>
-      <c r="F49" s="20"/>
-      <c r="G49" s="20"/>
-      <c r="H49" s="20"/>
-      <c r="I49" s="20"/>
-      <c r="J49" s="20"/>
-      <c r="K49" s="20"/>
-      <c r="L49" s="20"/>
-      <c r="M49" s="20"/>
-      <c r="N49" s="20"/>
-      <c r="O49" s="20"/>
-      <c r="P49" s="20"/>
-      <c r="Q49" s="20"/>
-      <c r="R49" s="20"/>
-      <c r="S49" s="20"/>
-      <c r="T49" s="20"/>
-      <c r="U49" s="20"/>
-      <c r="V49" s="20"/>
-      <c r="W49" s="20"/>
-      <c r="X49" s="20"/>
+      <c r="A49" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="B49" s="18"/>
+      <c r="C49" s="18"/>
+      <c r="D49" s="18"/>
+      <c r="E49" s="18"/>
+      <c r="F49" s="18"/>
+      <c r="G49" s="18"/>
+      <c r="H49" s="18"/>
+      <c r="I49" s="18"/>
+      <c r="J49" s="18"/>
+      <c r="K49" s="18"/>
+      <c r="L49" s="18"/>
+      <c r="M49" s="18"/>
+      <c r="N49" s="18"/>
+      <c r="O49" s="18"/>
+      <c r="P49" s="18"/>
+      <c r="Q49" s="18"/>
+      <c r="R49" s="18"/>
+      <c r="S49" s="18"/>
+      <c r="T49" s="18"/>
+      <c r="U49" s="18"/>
+      <c r="V49" s="18"/>
+      <c r="W49" s="18"/>
+      <c r="X49" s="18"/>
     </row>
     <row r="50" spans="1:24" ht="68.45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="20" t="s">
+      <c r="A50" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="B50" s="20"/>
-      <c r="C50" s="20"/>
-      <c r="D50" s="20"/>
-      <c r="E50" s="20"/>
-      <c r="F50" s="20"/>
-      <c r="G50" s="20"/>
-      <c r="H50" s="20"/>
-      <c r="I50" s="20"/>
-      <c r="J50" s="20"/>
-      <c r="K50" s="20"/>
-      <c r="L50" s="20"/>
-      <c r="M50" s="20"/>
-      <c r="N50" s="20"/>
-      <c r="O50" s="20"/>
-      <c r="P50" s="20"/>
-      <c r="Q50" s="20"/>
-      <c r="R50" s="20"/>
-      <c r="S50" s="20"/>
-      <c r="T50" s="20"/>
-      <c r="U50" s="20"/>
-      <c r="V50" s="20"/>
-      <c r="W50" s="20"/>
-      <c r="X50" s="20"/>
+      <c r="B50" s="18"/>
+      <c r="C50" s="18"/>
+      <c r="D50" s="18"/>
+      <c r="E50" s="18"/>
+      <c r="F50" s="18"/>
+      <c r="G50" s="18"/>
+      <c r="H50" s="18"/>
+      <c r="I50" s="18"/>
+      <c r="J50" s="18"/>
+      <c r="K50" s="18"/>
+      <c r="L50" s="18"/>
+      <c r="M50" s="18"/>
+      <c r="N50" s="18"/>
+      <c r="O50" s="18"/>
+      <c r="P50" s="18"/>
+      <c r="Q50" s="18"/>
+      <c r="R50" s="18"/>
+      <c r="S50" s="18"/>
+      <c r="T50" s="18"/>
+      <c r="U50" s="18"/>
+      <c r="V50" s="18"/>
+      <c r="W50" s="18"/>
+      <c r="X50" s="18"/>
     </row>
     <row r="51" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="20" t="s">
-        <v>81</v>
-      </c>
-      <c r="B51" s="20"/>
-      <c r="C51" s="20"/>
-      <c r="D51" s="20"/>
-      <c r="E51" s="20"/>
-      <c r="F51" s="20"/>
-      <c r="G51" s="20"/>
-      <c r="H51" s="20"/>
-      <c r="I51" s="20"/>
-      <c r="J51" s="20"/>
-      <c r="K51" s="20"/>
-      <c r="L51" s="20"/>
-      <c r="M51" s="20"/>
-      <c r="N51" s="20"/>
-      <c r="O51" s="20"/>
-      <c r="P51" s="20"/>
-      <c r="Q51" s="20"/>
-      <c r="R51" s="20"/>
-      <c r="S51" s="20"/>
-      <c r="T51" s="20"/>
-      <c r="U51" s="20"/>
-      <c r="V51" s="20"/>
-      <c r="W51" s="20"/>
-      <c r="X51" s="20"/>
+      <c r="A51" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="B51" s="18"/>
+      <c r="C51" s="18"/>
+      <c r="D51" s="18"/>
+      <c r="E51" s="18"/>
+      <c r="F51" s="18"/>
+      <c r="G51" s="18"/>
+      <c r="H51" s="18"/>
+      <c r="I51" s="18"/>
+      <c r="J51" s="18"/>
+      <c r="K51" s="18"/>
+      <c r="L51" s="18"/>
+      <c r="M51" s="18"/>
+      <c r="N51" s="18"/>
+      <c r="O51" s="18"/>
+      <c r="P51" s="18"/>
+      <c r="Q51" s="18"/>
+      <c r="R51" s="18"/>
+      <c r="S51" s="18"/>
+      <c r="T51" s="18"/>
+      <c r="U51" s="18"/>
+      <c r="V51" s="18"/>
+      <c r="W51" s="18"/>
+      <c r="X51" s="18"/>
     </row>
     <row r="52" spans="1:24" ht="26.45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="B52" s="20"/>
-      <c r="C52" s="20"/>
-      <c r="D52" s="20"/>
-      <c r="E52" s="20"/>
-      <c r="F52" s="20"/>
-      <c r="G52" s="20"/>
-      <c r="H52" s="20"/>
-      <c r="I52" s="20"/>
-      <c r="J52" s="20"/>
-      <c r="K52" s="20"/>
-      <c r="L52" s="20"/>
-      <c r="M52" s="20"/>
-      <c r="N52" s="20"/>
-      <c r="O52" s="20"/>
-      <c r="P52" s="20"/>
-      <c r="Q52" s="20"/>
-      <c r="R52" s="20"/>
-      <c r="S52" s="20"/>
-      <c r="T52" s="20"/>
-      <c r="U52" s="20"/>
-      <c r="V52" s="20"/>
-      <c r="W52" s="20"/>
-      <c r="X52" s="20"/>
+      <c r="A52" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="B52" s="18"/>
+      <c r="C52" s="18"/>
+      <c r="D52" s="18"/>
+      <c r="E52" s="18"/>
+      <c r="F52" s="18"/>
+      <c r="G52" s="18"/>
+      <c r="H52" s="18"/>
+      <c r="I52" s="18"/>
+      <c r="J52" s="18"/>
+      <c r="K52" s="18"/>
+      <c r="L52" s="18"/>
+      <c r="M52" s="18"/>
+      <c r="N52" s="18"/>
+      <c r="O52" s="18"/>
+      <c r="P52" s="18"/>
+      <c r="Q52" s="18"/>
+      <c r="R52" s="18"/>
+      <c r="S52" s="18"/>
+      <c r="T52" s="18"/>
+      <c r="U52" s="18"/>
+      <c r="V52" s="18"/>
+      <c r="W52" s="18"/>
+      <c r="X52" s="18"/>
     </row>
     <row r="53" spans="1:24" ht="26.45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="20" t="s">
-        <v>83</v>
-      </c>
-      <c r="B53" s="20"/>
-      <c r="C53" s="20"/>
-      <c r="D53" s="20"/>
-      <c r="E53" s="20"/>
-      <c r="F53" s="20"/>
-      <c r="G53" s="20"/>
-      <c r="H53" s="20"/>
-      <c r="I53" s="20"/>
-      <c r="J53" s="20"/>
-      <c r="K53" s="20"/>
-      <c r="L53" s="20"/>
-      <c r="M53" s="20"/>
-      <c r="N53" s="20"/>
-      <c r="O53" s="20"/>
-      <c r="P53" s="20"/>
-      <c r="Q53" s="20"/>
-      <c r="R53" s="20"/>
-      <c r="S53" s="20"/>
-      <c r="T53" s="20"/>
-      <c r="U53" s="20"/>
-      <c r="V53" s="20"/>
-      <c r="W53" s="20"/>
-      <c r="X53" s="20"/>
+      <c r="A53" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="B53" s="18"/>
+      <c r="C53" s="18"/>
+      <c r="D53" s="18"/>
+      <c r="E53" s="18"/>
+      <c r="F53" s="18"/>
+      <c r="G53" s="18"/>
+      <c r="H53" s="18"/>
+      <c r="I53" s="18"/>
+      <c r="J53" s="18"/>
+      <c r="K53" s="18"/>
+      <c r="L53" s="18"/>
+      <c r="M53" s="18"/>
+      <c r="N53" s="18"/>
+      <c r="O53" s="18"/>
+      <c r="P53" s="18"/>
+      <c r="Q53" s="18"/>
+      <c r="R53" s="18"/>
+      <c r="S53" s="18"/>
+      <c r="T53" s="18"/>
+      <c r="U53" s="18"/>
+      <c r="V53" s="18"/>
+      <c r="W53" s="18"/>
+      <c r="X53" s="18"/>
     </row>
     <row r="54" spans="1:24" ht="40.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="20" t="s">
-        <v>84</v>
-      </c>
-      <c r="B54" s="20"/>
-      <c r="C54" s="20"/>
-      <c r="D54" s="20"/>
-      <c r="E54" s="20"/>
-      <c r="F54" s="20"/>
-      <c r="G54" s="20"/>
-      <c r="H54" s="20"/>
-      <c r="I54" s="20"/>
-      <c r="J54" s="20"/>
-      <c r="K54" s="20"/>
-      <c r="L54" s="20"/>
-      <c r="M54" s="20"/>
-      <c r="N54" s="20"/>
-      <c r="O54" s="20"/>
-      <c r="P54" s="20"/>
-      <c r="Q54" s="20"/>
-      <c r="R54" s="20"/>
-      <c r="S54" s="20"/>
-      <c r="T54" s="20"/>
-      <c r="U54" s="20"/>
-      <c r="V54" s="20"/>
-      <c r="W54" s="20"/>
-      <c r="X54" s="20"/>
+      <c r="A54" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="B54" s="18"/>
+      <c r="C54" s="18"/>
+      <c r="D54" s="18"/>
+      <c r="E54" s="18"/>
+      <c r="F54" s="18"/>
+      <c r="G54" s="18"/>
+      <c r="H54" s="18"/>
+      <c r="I54" s="18"/>
+      <c r="J54" s="18"/>
+      <c r="K54" s="18"/>
+      <c r="L54" s="18"/>
+      <c r="M54" s="18"/>
+      <c r="N54" s="18"/>
+      <c r="O54" s="18"/>
+      <c r="P54" s="18"/>
+      <c r="Q54" s="18"/>
+      <c r="R54" s="18"/>
+      <c r="S54" s="18"/>
+      <c r="T54" s="18"/>
+      <c r="U54" s="18"/>
+      <c r="V54" s="18"/>
+      <c r="W54" s="18"/>
+      <c r="X54" s="18"/>
     </row>
     <row r="55" spans="1:24" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="20" t="s">
-        <v>85</v>
-      </c>
-      <c r="B55" s="23"/>
-      <c r="C55" s="23"/>
-      <c r="D55" s="23"/>
-      <c r="E55" s="23"/>
-      <c r="F55" s="23"/>
-      <c r="G55" s="23"/>
-      <c r="H55" s="23"/>
-      <c r="I55" s="23"/>
-      <c r="J55" s="23"/>
-      <c r="K55" s="23"/>
-      <c r="L55" s="23"/>
-      <c r="M55" s="23"/>
-      <c r="N55" s="23"/>
-      <c r="O55" s="23"/>
-      <c r="P55" s="23"/>
-      <c r="Q55" s="23"/>
-      <c r="R55" s="23"/>
-      <c r="S55" s="23"/>
-      <c r="T55" s="23"/>
-      <c r="U55" s="23"/>
-      <c r="V55" s="23"/>
-      <c r="W55" s="23"/>
-      <c r="X55" s="23"/>
+      <c r="A55" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="B55" s="21"/>
+      <c r="C55" s="21"/>
+      <c r="D55" s="21"/>
+      <c r="E55" s="21"/>
+      <c r="F55" s="21"/>
+      <c r="G55" s="21"/>
+      <c r="H55" s="21"/>
+      <c r="I55" s="21"/>
+      <c r="J55" s="21"/>
+      <c r="K55" s="21"/>
+      <c r="L55" s="21"/>
+      <c r="M55" s="21"/>
+      <c r="N55" s="21"/>
+      <c r="O55" s="21"/>
+      <c r="P55" s="21"/>
+      <c r="Q55" s="21"/>
+      <c r="R55" s="21"/>
+      <c r="S55" s="21"/>
+      <c r="T55" s="21"/>
+      <c r="U55" s="21"/>
+      <c r="V55" s="21"/>
+      <c r="W55" s="21"/>
+      <c r="X55" s="21"/>
     </row>
     <row r="56" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="20" t="s">
-        <v>86</v>
-      </c>
-      <c r="B56" s="20"/>
-      <c r="C56" s="20"/>
-      <c r="D56" s="20"/>
-      <c r="E56" s="20"/>
-      <c r="F56" s="20"/>
-      <c r="G56" s="20"/>
-      <c r="H56" s="20"/>
-      <c r="I56" s="20"/>
-      <c r="J56" s="20"/>
-      <c r="K56" s="20"/>
-      <c r="L56" s="20"/>
-      <c r="M56" s="20"/>
-      <c r="N56" s="20"/>
-      <c r="O56" s="20"/>
-      <c r="P56" s="20"/>
-      <c r="Q56" s="20"/>
-      <c r="R56" s="20"/>
-      <c r="S56" s="20"/>
-      <c r="T56" s="20"/>
-      <c r="U56" s="20"/>
-      <c r="V56" s="20"/>
-      <c r="W56" s="20"/>
-      <c r="X56" s="20"/>
+      <c r="A56" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="B56" s="18"/>
+      <c r="C56" s="18"/>
+      <c r="D56" s="18"/>
+      <c r="E56" s="18"/>
+      <c r="F56" s="18"/>
+      <c r="G56" s="18"/>
+      <c r="H56" s="18"/>
+      <c r="I56" s="18"/>
+      <c r="J56" s="18"/>
+      <c r="K56" s="18"/>
+      <c r="L56" s="18"/>
+      <c r="M56" s="18"/>
+      <c r="N56" s="18"/>
+      <c r="O56" s="18"/>
+      <c r="P56" s="18"/>
+      <c r="Q56" s="18"/>
+      <c r="R56" s="18"/>
+      <c r="S56" s="18"/>
+      <c r="T56" s="18"/>
+      <c r="U56" s="18"/>
+      <c r="V56" s="18"/>
+      <c r="W56" s="18"/>
+      <c r="X56" s="18"/>
     </row>
     <row r="57" spans="1:24" ht="78" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A57" s="20" t="s">
-        <v>87</v>
-      </c>
-      <c r="B57" s="20"/>
-      <c r="C57" s="20"/>
-      <c r="D57" s="20"/>
-      <c r="E57" s="20"/>
-      <c r="F57" s="20"/>
-      <c r="G57" s="20"/>
-      <c r="H57" s="20"/>
-      <c r="I57" s="20"/>
-      <c r="J57" s="20"/>
-      <c r="K57" s="20"/>
-      <c r="L57" s="20"/>
-      <c r="M57" s="20"/>
-      <c r="N57" s="20"/>
-      <c r="O57" s="20"/>
-      <c r="P57" s="20"/>
-      <c r="Q57" s="20"/>
-      <c r="R57" s="20"/>
-      <c r="S57" s="20"/>
-      <c r="T57" s="20"/>
-      <c r="U57" s="20"/>
-      <c r="V57" s="20"/>
-      <c r="W57" s="20"/>
-      <c r="X57" s="20"/>
+      <c r="A57" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="B57" s="18"/>
+      <c r="C57" s="18"/>
+      <c r="D57" s="18"/>
+      <c r="E57" s="18"/>
+      <c r="F57" s="18"/>
+      <c r="G57" s="18"/>
+      <c r="H57" s="18"/>
+      <c r="I57" s="18"/>
+      <c r="J57" s="18"/>
+      <c r="K57" s="18"/>
+      <c r="L57" s="18"/>
+      <c r="M57" s="18"/>
+      <c r="N57" s="18"/>
+      <c r="O57" s="18"/>
+      <c r="P57" s="18"/>
+      <c r="Q57" s="18"/>
+      <c r="R57" s="18"/>
+      <c r="S57" s="18"/>
+      <c r="T57" s="18"/>
+      <c r="U57" s="18"/>
+      <c r="V57" s="18"/>
+      <c r="W57" s="18"/>
+      <c r="X57" s="18"/>
     </row>
     <row r="58" spans="1:24" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A58" s="26" t="s">
-        <v>88</v>
-      </c>
-      <c r="B58" s="26"/>
-      <c r="C58" s="26"/>
-      <c r="D58" s="26"/>
-      <c r="E58" s="26"/>
-      <c r="F58" s="26"/>
-      <c r="G58" s="26"/>
-      <c r="H58" s="26"/>
-      <c r="I58" s="26"/>
-      <c r="J58" s="26"/>
-      <c r="K58" s="26"/>
-      <c r="L58" s="26"/>
-      <c r="M58" s="26"/>
-      <c r="N58" s="26"/>
-      <c r="O58" s="26"/>
-      <c r="P58" s="26"/>
-      <c r="Q58" s="26"/>
-      <c r="R58" s="26"/>
-      <c r="S58" s="26"/>
-      <c r="T58" s="26"/>
-      <c r="U58" s="26"/>
-      <c r="V58" s="26"/>
-      <c r="W58" s="26"/>
-      <c r="X58" s="26"/>
+      <c r="A58" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="B58" s="24"/>
+      <c r="C58" s="24"/>
+      <c r="D58" s="24"/>
+      <c r="E58" s="24"/>
+      <c r="F58" s="24"/>
+      <c r="G58" s="24"/>
+      <c r="H58" s="24"/>
+      <c r="I58" s="24"/>
+      <c r="J58" s="24"/>
+      <c r="K58" s="24"/>
+      <c r="L58" s="24"/>
+      <c r="M58" s="24"/>
+      <c r="N58" s="24"/>
+      <c r="O58" s="24"/>
+      <c r="P58" s="24"/>
+      <c r="Q58" s="24"/>
+      <c r="R58" s="24"/>
+      <c r="S58" s="24"/>
+      <c r="T58" s="24"/>
+      <c r="U58" s="24"/>
+      <c r="V58" s="24"/>
+      <c r="W58" s="24"/>
+      <c r="X58" s="24"/>
     </row>
     <row r="59" spans="1:24" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A59" s="20" t="s">
-        <v>89</v>
-      </c>
-      <c r="B59" s="20"/>
-      <c r="C59" s="20"/>
-      <c r="D59" s="20"/>
-      <c r="E59" s="20"/>
-      <c r="F59" s="20"/>
-      <c r="G59" s="20"/>
-      <c r="H59" s="20"/>
-      <c r="I59" s="20"/>
-      <c r="J59" s="20"/>
-      <c r="K59" s="20"/>
-      <c r="L59" s="20"/>
-      <c r="M59" s="20"/>
-      <c r="N59" s="20"/>
-      <c r="O59" s="20"/>
-      <c r="P59" s="20"/>
-      <c r="Q59" s="20"/>
-      <c r="R59" s="20"/>
-      <c r="S59" s="20"/>
-      <c r="T59" s="20"/>
-      <c r="U59" s="20"/>
-      <c r="V59" s="20"/>
-      <c r="W59" s="20"/>
-      <c r="X59" s="20"/>
+      <c r="A59" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="B59" s="18"/>
+      <c r="C59" s="18"/>
+      <c r="D59" s="18"/>
+      <c r="E59" s="18"/>
+      <c r="F59" s="18"/>
+      <c r="G59" s="18"/>
+      <c r="H59" s="18"/>
+      <c r="I59" s="18"/>
+      <c r="J59" s="18"/>
+      <c r="K59" s="18"/>
+      <c r="L59" s="18"/>
+      <c r="M59" s="18"/>
+      <c r="N59" s="18"/>
+      <c r="O59" s="18"/>
+      <c r="P59" s="18"/>
+      <c r="Q59" s="18"/>
+      <c r="R59" s="18"/>
+      <c r="S59" s="18"/>
+      <c r="T59" s="18"/>
+      <c r="U59" s="18"/>
+      <c r="V59" s="18"/>
+      <c r="W59" s="18"/>
+      <c r="X59" s="18"/>
     </row>
     <row r="60" spans="1:24" ht="39" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A60" s="20" t="s">
-        <v>90</v>
-      </c>
-      <c r="B60" s="20"/>
-      <c r="C60" s="20"/>
-      <c r="D60" s="20"/>
-      <c r="E60" s="20"/>
-      <c r="F60" s="20"/>
-      <c r="G60" s="20"/>
-      <c r="H60" s="20"/>
-      <c r="I60" s="20"/>
-      <c r="J60" s="20"/>
-      <c r="K60" s="20"/>
-      <c r="L60" s="20"/>
-      <c r="M60" s="20"/>
-      <c r="N60" s="20"/>
-      <c r="O60" s="20"/>
-      <c r="P60" s="20"/>
-      <c r="Q60" s="20"/>
-      <c r="R60" s="20"/>
-      <c r="S60" s="20"/>
-      <c r="T60" s="20"/>
-      <c r="U60" s="20"/>
-      <c r="V60" s="20"/>
-      <c r="W60" s="20"/>
-      <c r="X60" s="20"/>
+      <c r="A60" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="B60" s="18"/>
+      <c r="C60" s="18"/>
+      <c r="D60" s="18"/>
+      <c r="E60" s="18"/>
+      <c r="F60" s="18"/>
+      <c r="G60" s="18"/>
+      <c r="H60" s="18"/>
+      <c r="I60" s="18"/>
+      <c r="J60" s="18"/>
+      <c r="K60" s="18"/>
+      <c r="L60" s="18"/>
+      <c r="M60" s="18"/>
+      <c r="N60" s="18"/>
+      <c r="O60" s="18"/>
+      <c r="P60" s="18"/>
+      <c r="Q60" s="18"/>
+      <c r="R60" s="18"/>
+      <c r="S60" s="18"/>
+      <c r="T60" s="18"/>
+      <c r="U60" s="18"/>
+      <c r="V60" s="18"/>
+      <c r="W60" s="18"/>
+      <c r="X60" s="18"/>
     </row>
     <row r="61" spans="1:24" ht="80.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A61" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="B61" s="20"/>
-      <c r="C61" s="20"/>
-      <c r="D61" s="20"/>
-      <c r="E61" s="20"/>
-      <c r="F61" s="20"/>
-      <c r="G61" s="20"/>
-      <c r="H61" s="20"/>
-      <c r="I61" s="20"/>
-      <c r="J61" s="20"/>
-      <c r="K61" s="20"/>
-      <c r="L61" s="20"/>
-      <c r="M61" s="20"/>
-      <c r="N61" s="20"/>
-      <c r="O61" s="20"/>
-      <c r="P61" s="20"/>
-      <c r="Q61" s="20"/>
-      <c r="R61" s="20"/>
-      <c r="S61" s="20"/>
-      <c r="T61" s="20"/>
-      <c r="U61" s="20"/>
-      <c r="V61" s="20"/>
-      <c r="W61" s="20"/>
-      <c r="X61" s="20"/>
+      <c r="A61" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="B61" s="18"/>
+      <c r="C61" s="18"/>
+      <c r="D61" s="18"/>
+      <c r="E61" s="18"/>
+      <c r="F61" s="18"/>
+      <c r="G61" s="18"/>
+      <c r="H61" s="18"/>
+      <c r="I61" s="18"/>
+      <c r="J61" s="18"/>
+      <c r="K61" s="18"/>
+      <c r="L61" s="18"/>
+      <c r="M61" s="18"/>
+      <c r="N61" s="18"/>
+      <c r="O61" s="18"/>
+      <c r="P61" s="18"/>
+      <c r="Q61" s="18"/>
+      <c r="R61" s="18"/>
+      <c r="S61" s="18"/>
+      <c r="T61" s="18"/>
+      <c r="U61" s="18"/>
+      <c r="V61" s="18"/>
+      <c r="W61" s="18"/>
+      <c r="X61" s="18"/>
     </row>
     <row r="62" spans="1:24" ht="86.1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A62" s="20" t="s">
-        <v>92</v>
-      </c>
-      <c r="B62" s="20"/>
-      <c r="C62" s="20"/>
-      <c r="D62" s="20"/>
-      <c r="E62" s="20"/>
-      <c r="F62" s="20"/>
-      <c r="G62" s="20"/>
-      <c r="H62" s="20"/>
-      <c r="I62" s="20"/>
-      <c r="J62" s="20"/>
-      <c r="K62" s="20"/>
-      <c r="L62" s="20"/>
-      <c r="M62" s="20"/>
-      <c r="N62" s="20"/>
-      <c r="O62" s="20"/>
-      <c r="P62" s="20"/>
-      <c r="Q62" s="20"/>
-      <c r="R62" s="20"/>
-      <c r="S62" s="20"/>
-      <c r="T62" s="20"/>
-      <c r="U62" s="20"/>
-      <c r="V62" s="20"/>
-      <c r="W62" s="20"/>
-      <c r="X62" s="20"/>
+      <c r="A62" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="B62" s="18"/>
+      <c r="C62" s="18"/>
+      <c r="D62" s="18"/>
+      <c r="E62" s="18"/>
+      <c r="F62" s="18"/>
+      <c r="G62" s="18"/>
+      <c r="H62" s="18"/>
+      <c r="I62" s="18"/>
+      <c r="J62" s="18"/>
+      <c r="K62" s="18"/>
+      <c r="L62" s="18"/>
+      <c r="M62" s="18"/>
+      <c r="N62" s="18"/>
+      <c r="O62" s="18"/>
+      <c r="P62" s="18"/>
+      <c r="Q62" s="18"/>
+      <c r="R62" s="18"/>
+      <c r="S62" s="18"/>
+      <c r="T62" s="18"/>
+      <c r="U62" s="18"/>
+      <c r="V62" s="18"/>
+      <c r="W62" s="18"/>
+      <c r="X62" s="18"/>
     </row>
     <row r="64" spans="1:24" ht="13.15" x14ac:dyDescent="0.4">
       <c r="A64" t="s">
-        <v>93</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>